<commit_message>
feat(news): publish 2026-10-19 daily brief
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-18-en.xlsx
+++ b/docs/exports/week-2026-10-18-en.xlsx
@@ -538,21 +538,21 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Kumamoto fab approval and Taiwanese equipment-service acquisition authorization
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Japan approved JASM’s revised second-fab plan on October 16, while Taiwan Mask changed the proposed TCK buyer to the parent. Fab construction and unconfirmed acquisition closing represent separate process-build and local-service milestones.</t>
+            <t xml:space="preserve">Vietnam–EFTA signature sets out equipment and investment rules, subject to effective terms
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Vietnam and the four EFTA states signed in Hanoi on October 18, covering goods, services, investment, origin and procurement. Machinery and electrical goods are established trade categories, while effective dates and product treatment cannot be established from signature alone.</t>
           </r>
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
     </row>
     <row r="4" ht="82" customHeight="1">
@@ -570,16 +570,16 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Malaysia’s six innovations span storage, industrial control and power
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>The October 16 launches include AI processors, storage, FPGA and automotive/satellite power control. The minister’s RM300 million combined sales potential has no stated period, with customer qualification and production volumes undisclosed.</t>
+            <t xml:space="preserve">Kumamoto fab approval and local equipment-service acquisition authorization
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Professional reports describe Japan’s October 16 approval of JASM’s initial 3nm phase, while Taiwan Mask changed the proposed TCK buyer to the parent. Wafer capacity remains planned and the acquisition has no confirmed closing, with limited direct access to the underlying approval and filing.</t>
           </r>
         </is>
       </c>
@@ -587,7 +587,7 @@
         <v>46311</v>
       </c>
     </row>
-    <row r="5" ht="82" customHeight="1">
+    <row r="5" ht="102" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>03</t>
@@ -602,21 +602,21 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Vietnamese rolling line reaches core-equipment contract stage
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>VinMetal and Danieli signed the core-equipment contract on October 15 for Ha Tinh’s Vung Ang Economic Zone. Above 700,000 tonnes is one line’s annual design capacity; delivery, start-up and customer-acceptance schedules are undisclosed.</t>
+            <t xml:space="preserve">Foxconn’s proposed half-stake in Mitsubishi Electric Mobility covers powertrains and control
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>The October 16 agreement sets ¥115 billion for 50%, against total equity value of ¥230 billion. Closing is planned for October 1, 2027 subject to approvals and conditions, without incremental shipments or factory-output figures.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="6" ht="82" customHeight="1">
@@ -634,53 +634,55 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Thai materials land and Johor smart campus remain planning-stage projects
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>LCY Technology approved Thai subsidiary land plans on October 16 with site and price pending; reports the same day described Genting and Huawei’s 430-acre Kulai campus plan. Neither provides verified new production, tenant or paid-investment figures.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n">
+            <t xml:space="preserve">Taiwanese storage, fuel logistics and wind works have separate completion milestones
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Foxconn’s partners announced a planned 306 kWh cabinet and H1 2027 supply target on October 16; MOEA said October 18 that CPC began next-quarter fuel procurement. Four installed offshore turbines are a reported official figure, distinct from grid connection or a final loan-repayment settlement.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Oct 16, Oct 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="102" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Singapore electronics exports and Malaysian chip launches describe shipments and development
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Singapore reported September NODX growth of 68.4% and Taiwan-bound growth of 96.9% on October 16, with ship-structure base effects in the aggregate. Malaysia launched six domestic innovations the same day; RM300 million sales potential lacks a period, and launch-venue reports differ.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
         <v>46311</v>
-      </c>
-    </row>
-    <row r="7" ht="82" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Vietnam sets 2027 targets and a 2026 full-year trade estimate
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>The government presented next-year targets to parliament on October 17: at least 10% GDP growth, CPI around 4.5% and 8.6% productivity growth. Estimated 2026 merchandise trade of US$1.11 trillion and the targets must be distinguished from completed results.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>46312</v>
       </c>
     </row>
   </sheetData>
@@ -699,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -737,7 +739,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="214" customHeight="1">
+    <row r="3" ht="230" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>01</t>
@@ -752,6 +754,43 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
+            <t xml:space="preserve">Vietnam signs FTA with four EFTA states covering industrial goods, origin and investment rules
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Vietnam and Switzerland, Norway, Iceland and Liechtenstein signed an FTA in Hanoi on October 18, covering goods, services, origin, investment and procurement. Electrical and mechanical machinery already feature in bilateral trade; signature does not establish immediate duty-free treatment for every product. EFTA identifies electrical and mechanical machinery in existing bilateral goods trade. MOIT lists tariffs, technical barriers, customs procedures and investment among the agreement’s provisions, without naming suppliers or newly committed production lines. Negotiations concluded on July 2, followed by signature on October 18. EFTA’s linked chapter factsheet remains the July version and describes product-specific origin rules; signature, domestic procedures and effective preferences are separate stages. The inspected announcements do not establish an entry-into-force date or product-level preference schedules. Equipment tariff, origin and certification treatment depends on the definitive agreement and schedules. Location: Signing location: Hanoi, Vietnam. The inspected official announcements do not identify the venue.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>46313</v>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>For precision-power and measurement/control suppliers, the relevant link is cross-border trade in Vietnamese factory equipment and test products. Questions concern tariff classification, origin and certification under the effective text; no customer purchasing data establish incremental orders from signature alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="214" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
             <t xml:space="preserve">Follow-up: Japan approves revised JASM Kumamoto plan with 6,000 3nm wafers a month initially
 </t>
           </r>
@@ -762,43 +801,6 @@
               <sz val="11"/>
             </rPr>
             <t>Reuters and CNA report that Japan approved a revised plan for TSMC subsidiary JASM’s second Kumamoto fab on October 16, with initial capacity of 6,000 3nm wafers a month. Approval is the new development; the technology shift was announced in February, and the fab remains under construction. JASM is TSMC’s Japanese manufacturing subsidiary, and the second fab adjoins its existing Kumamoto facility. The approval concerns wafer processing and tool deployment; it contains no new HBM, packaging/test or server shipment data. CNA reports production is planned for late 2028. The earlier 48,000-wafer monthly plan covered a different process mix and build scope, so it is not a comparable base for calculating a capacity reduction. The METI approval document was not directly obtained; capacity and timing rely on professional reporting. Tool lists, yields and actual production capability remain undisclosed. Location: Project site: JASM’s second fab in Kumamoto Prefecture, Japan, adjacent to its first fab.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>46311</v>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>For precision-power and measurement suppliers serving etch and deposition, the relevant customers are fabs and process-tool makers. Questions concern 3nm tool qualification, installation and acceptance timing; planned wafer capacity alone cannot establish equipment purchases or supplier orders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="194" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Follow-up: Taiwan Mask names parent as proposed TCK buyer, with a ¥750 million ceiling
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Taiwan Mask’s board on October 16 authorized its chairman to acquire all of Kumamoto equipment-service company TCK for up to ¥750 million, about NT$160 million according to CNA. The proposed buyer changed from subsidiary Guang Ju Holdings in July to Taiwan Mask itself; the confirmed development is board authorization. Taiwan Mask supplies semiconductor masks; Kumamoto-based TCK provides equipment assembly and engineering services. The filing concerns shares in a service business and gives no additional wafer, packaging or test capacity. ¥750 million is an authorization ceiling. CNA’s NT$160 million equivalent is approximate rather than paid consideration; exchange rates and final terms can change the Taiwan-dollar amount. The filing was checked through Cnyes’s reproduction, without direct retrieval from MOPS. The final price, closing date and integration details remain undisclosed. Location: Target location: T.C.K Corporation, Kumamoto City, Japan. The board meeting venue was not disclosed.</t>
           </r>
         </is>
       </c>
@@ -807,11 +809,11 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>For process-power and measurement/control suppliers, equipment assembly and local engineering relate to installation, service and acceptance support. Relevant checks include TCK’s tool scope, customer authorizations and quality processes; the share-acquisition authorization does not establish new supply relationships.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="278" customHeight="1">
+          <t>For precision-power and measurement suppliers serving etch and deposition, the relevant customers are fabs and process-tool makers. Questions concern 3nm tool qualification, installation and acceptance timing; planned wafer capacity alone cannot establish equipment purchases or supplier orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="194" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>03</t>
@@ -826,16 +828,16 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Malaysia launches six domestic chip innovations spanning AI storage, industrial FPGA and power control
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Malaysia launched six domestic semiconductor innovations at AiSEM in Kuala Lumpur on October 16, spanning AI processors, storage, programmable logic and power control. The economy minister cited combined sales potential of RM300 million without an achievement period; production shipment figures were not provided. The Edge lists SkyeChip’s MARS1000 AI processor, MaiStorage’s aiDAPTIV+ storage solution, SiliconX’s industrial/automotive FPGA, Infinecs’ automotive power regulator, Weeroc Space’s satellite power controller and Alphaswift’s FC Mini flight controller. Applications extend to factories, computers, servers, vehicles and aerospace. The state-government English report quotes the chief minister saying Weeroc Space’s GaN power chip completed its second tape-out. Tape-out, launch, customer qualification and volume production are separate milestones; RM300 million is the minister’s combined commercial-potential estimate, with no annual revenue or signed orders disclosed. Customer qualification, volume-production timing, sales bases and the period for realizing the combined potential remain undisclosed. Event reports differ between Grand Hyatt and KLCC as the launch venue. Location: Event city: Kuala Lumpur, Malaysia. The organizer schedule, state-government English report and Malay Mail identify Grand Hyatt; the state-government Malay report identifies KLCC, leaving a launch-venue discrepancy.</t>
+            <t xml:space="preserve">Follow-up: Taiwan Mask names parent as proposed TCK buyer, with a ¥750 million ceiling
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Taiwan Mask’s board on October 16 authorized its chairman to acquire all of Kumamoto equipment-service company TCK for up to ¥750 million, about NT$160 million according to CNA. The proposed buyer changed from subsidiary Guang Ju Holdings in July to Taiwan Mask itself; the confirmed development is board authorization. Taiwan Mask supplies semiconductor masks; Kumamoto-based TCK provides equipment assembly and engineering services. The filing concerns shares in a service business and gives no additional wafer, packaging or test capacity. ¥750 million is an authorization ceiling. CNA’s NT$160 million equivalent is approximate rather than paid consideration; exchange rates and final terms can change the Taiwan-dollar amount. The filing was checked through Cnyes’s reproduction, without direct retrieval from MOPS. The final price, closing date and integration details remain undisclosed. Location: Target location: T.C.K Corporation, Kumamoto City, Japan. The board meeting venue was not disclosed.</t>
           </r>
         </is>
       </c>
@@ -844,11 +846,11 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>For precision-power, measurement and control suppliers, automotive regulation, satellite power control and factory logic are specific related applications. Questions concern each product’s tape-out, test and customer-validation stage; combined sales potential cannot establish equipment demand or orders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="210" customHeight="1">
+          <t>For process-power and measurement/control suppliers, equipment assembly and local engineering relate to installation, service and acceptance support. Relevant checks include TCK’s tool scope, customer authorizations and quality processes; the share-acquisition authorization does not establish new supply relationships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="246" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>04</t>
@@ -863,29 +865,29 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">VinMetal signs Danieli rolling-line contract for over 700,000 tonnes a year in Ha Tinh
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>VinMetal and Italy’s Danieli signed a contract in Hanoi on October 15 for core rail and structural-steel rolling equipment at VinMetal’s Ha Tinh project. Vingroup states designed annual capacity above 700,000 tonnes, with design, manufacturing, supply and commissioning in scope; price and start-up date remain undisclosed. Danieli’s scope includes core rolling equipment and commissioning, with rail finishing and head-hardening technology described in the release. These processes establish final dimensions, properties and quality; power, measurement and control-system suppliers were not named. Above 700,000 tonnes is the annual design capacity of this rail and structural-steel line, rather than the entire complex or produced/sold tonnage. No like-for-like prior capacity was supplied, so no growth rate is calculated. Equipment delivery, commissioning and customer-acceptance schedules, actual output and contract consideration remain undisclosed. Location: Signing location: Hanoi, Vietnam. Project site: VinMetal’s factory in Vung Ang Economic Zone, Ha Tinh Province, Vietnam.</t>
+            <t xml:space="preserve">Foxconn proposes ¥115 billion for 50% of Mitsubishi Electric Mobility, with closing planned in 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Foxconn and Mitsubishi Electric announced on October 16 that Foxconn subsidiary Lin Yin plans to acquire 50% of Mitsubishi Electric Mobility for ¥115 billion and jointly operate the automotive-equipment business. Closing is planned for October 1, 2027, subject to regulatory approvals and contractual conditions. Mitsubishi Electric Mobility handles Mitsubishi Electric’s automotive-equipment business. The joint release identifies electric powertrains, software and vehicle control, with Japan-developed EV platforms as a stated direction. These are cooperation plans rather than new semiconductor-process or data-center capacity announcements. The agreement states enterprise value of ¥320 billion and equity value of ¥230 billion; the ¥115 billion consideration represents 50% of equity value. Enterprise value, total equity value and a partial-stake price have different scopes. Figures remain in the announced yen, without an independently assumed Taiwan-dollar conversion. Closing remains conditional on regulatory approvals and contractual requirements. Incremental orders, integrated production volumes and new-factory start-up schedules were not disclosed. Location: Announcement cities: Taipei, Taiwan, and Tokyo, Japan. No new factory site is specified.</t>
           </r>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>For industrial power-conversion and measurement/control suppliers, rolling, finishing and thermal processing involve process control and quality verification. Questions concern Danieli’s equipment interfaces, site power conditions and acceptance requirements; delivery schedules and subcontractor lists are still insufficient to establish specific equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="162" customHeight="1">
+          <t>For power-conversion and measurement/control suppliers, the relevant products are electric powertrains, vehicle control and their validation systems. Questions concern platform electrical specifications, supplier qualification and production acceptance; the transaction is conditional and contains no equipment purchasing or customer-order data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="226" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>05</t>
@@ -900,16 +902,16 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">LCY Technology approves Thai subsidiary land purchase; site and price remain pending
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>LCY Technology announced on October 16 that its board approved an industrial-land purchase by LCY Technology (Thailand). The company makes electrolytic copper foil for PCBs and copper-clad laminates; the seller, price, city and added capacity were not disclosed. CNA identifies PCB and copper-clad-laminate uses, linking materials and boards to electronic systems. The filing approves land only and does not specify future grades, applications or customers, leaving any dedicated AI-server line unconfirmed. The original filing was checked through a reproduction. The precise site, counterparty, land price, construction and production schedules remain undisclosed. Location: Project country: Thailand, industrial-estate land. The city and estate name have not been disclosed.</t>
+            <t xml:space="preserve">Foxconn-led storage partnership plans a 306 kWh cabinet and supply in 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Foxconn and Taiwanese storage partners announced an agreement during Energy Taiwan on October 16 for a planned 306 kWh domestically developed behind-the-meter battery cabinet. They target certification and supply in the first half of 2027, and 100 MWh of cumulative deployment in 2027; both remain targets. Foxconn supplies domestic cells, while partners including Rich Electric, Billion Watts and NoonSpare combine manufacturing, engineering and customer service. The company describes standalone DC battery cabinets or systems integrated with a power-conversion system (PCS) and energy-management system (EMS), for commercial/industrial storage and demand management. The 306 kWh figure describes planned energy per cabinet; 100 MWh describes cumulative market deployment targeted for 2027, a different scope and period. Development is planned in 2026, followed by certification and supply in H1 2027, without a comparable installed base. Completed certification, commercial supply and accepted installations have not been disclosed. The 306 kWh figure is stored energy, not PCS output power, which was not stated. Location: Exhibition venue: Taipei Nangang Exhibition Center Hall 1, Taiwan, October 14–16. The release does not specify a separate signing room.</t>
           </r>
         </is>
       </c>
@@ -918,11 +920,11 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>For process-power and industrial-measurement suppliers, copper-foil production can involve electrochemical processing, quality measurement and site power, but this announcement establishes land authorization only. Questions concern product specifications, engineering scope and equipment acceptance; construction data do not yet support an equipment-order assessment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="178" customHeight="1">
+          <t>For power-conversion and measurement/control suppliers, relevant customers include battery-system integrators and industrial users, with PCS/EMS interfaces and site acceptance in scope. Questions concern rated power, communications and certification; the energy specification and deployment target do not establish ordered converter quantities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="230" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>06</t>
@@ -937,62 +939,136 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Genting and Huawei plan a 430-acre Johor smart campus without a new investment figure
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Reports on October 16 said Genting Property and Huawei Malaysia had signed a master-planning agreement covering a 430-acre smart campus in Kulai, Johor. This is a planning collaboration, with no signed tenants, data-center MW capacity or incremental FDI amount disclosed. Bernama quotes the company saying Huawei will contribute AI and smart-campus planning expertise, with agricultural technology and energy management also mentioned. The 430 acres are planned campus land, with no basis for conversion to data-hall floor area or energized capacity. The agreement text was not obtained. Reports differ by a day on the statement date; construction timing, actual investment, tenants and power capacity remain undisclosed. Location: Project site: Johor Tech Smart City, Kulai, Johor, Malaysia. Signing-event venue: Shenzhen Longgang International Art Centre, China; the exact signing date was not disclosed.</t>
+            <t xml:space="preserve">MOEA reports four turbines installed at Taipower Phase II as payment and loan disputes continue
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Taiwan’s MOEA said on October 18 that a batch of three turbines was installed at Taipower’s offshore Phase II project on October 16, bringing the cumulative total to four. MOEA said supervised payments cover subcontractors amid Fuwei’s syndicated-loan dispute; installation progress is separate from a final repayment arrangement. MOEA said Fuwei requested Taipower take over turbine installation, with further work subject to weather and safety conditions. Turbine installation is distinct from electrical testing, grid connection and commercial operation, whose dates were not provided. MOEA described Taipower as a third party to Fuwei’s loan dispute and said it was communicating with the lenders. This describes the ministry’s position on payment mechanisms rather than contractual, lender or court findings on rights and obligations. Installation figures rely on CNA’s report of MOEA’s statement, without direct site-acceptance records or contracts. Grid-connection timing, final liability and bank-repayment arrangements remain unconfirmed. Location: Project: Taipower offshore Phase II, Taiwan. This statement does not provide precise worksite coordinates.</t>
           </r>
         </is>
       </c>
       <c r="C8" s="6" t="n">
+        <v>46313</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>For industrial-power and measurement/control suppliers, relevant stages include post-installation electrical tests, control validation and grid acceptance. Questions concern acceptance criteria and payment mechanisms for equipment and subcontractors; installation counts do not establish cash collection without contracts and final repayment arrangements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="146" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">MOEA says year-end fuel supply is secured and CPC has begun Q1 2027 procurement
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Taiwan’s MOEA said on October 18 that CPC was arranging alternative fuel sources and shipping schedules and had begun procurement for Q1 2027, with supply assessed as secured through year-end. This is an official assessment of fuel logistics, without detailed sources, cargoes, inventories or purchase prices. MOEA describes CPC sourcing alternatives and maintaining reserves, with Taipower handling generation and electricity dispatch. The statement does not announce a new industrial tariff or guarantee a specific volume to any factory, park or data center. Supply sufficiency is MOEA’s assessment. Cargo-level procurement and arrival records, user outage rates and final power costs were not provided for independent verification.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>46313</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>For industrial/data-center-power and measurement/control suppliers, fuel logistics provide context for customer power conditions. Questions concern site-specific grid access, power quality and acceptance criteria; a national supply assessment does not establish a particular site’s reliability or equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="278" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Malaysia launches six domestic chip innovations spanning AI storage, industrial FPGA and power control
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Malaysia launched six domestic semiconductor innovations at AiSEM in Kuala Lumpur on October 16, spanning AI processors, storage, programmable logic and power control. The economy minister cited combined sales potential of RM300 million without an achievement period; production shipment figures were not provided. The Edge lists SkyeChip’s MARS1000 AI processor, MaiStorage’s aiDAPTIV+ storage solution, SiliconX’s industrial/automotive FPGA, Infinecs’ automotive power regulator, Weeroc Space’s satellite power controller and Alphaswift’s FC Mini flight controller. Applications extend to factories, computers, servers, vehicles and aerospace. The state-government English report quotes the chief minister saying Weeroc Space’s GaN power chip completed its second tape-out. Tape-out, launch, customer qualification and volume production are separate milestones; RM300 million is the minister’s combined commercial-potential estimate, with no annual revenue or signed orders disclosed. Customer qualification, volume-production timing, sales bases and the period for realizing the combined potential remain undisclosed. Event reports differ between Grand Hyatt and KLCC as the launch venue. Location: Event city: Kuala Lumpur, Malaysia. The organizer schedule, state-government English report and Malay Mail identify Grand Hyatt; the state-government Malay report identifies KLCC, leaving a launch-venue discrepancy.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
         <v>46311</v>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>For data-center/industrial-power and measurement/control suppliers, campus energy management is a related application, but the evidence establishes master planning only. Questions concern actual tenants, distribution design and data-hall capacity; land area cannot establish power-equipment volumes or purchasing dates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="194" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Vietnam proposes at least 10% growth for 2027 and estimates 2026 trade at US$1.11 trillion
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Vietnam’s government presented 2027 targets to parliament on October 17: GDP growth of at least 10%, CPI around 4.5% and labor-productivity growth of 8.6%. Its report also estimates 2026 merchandise trade at US$1.11 trillion; the targets and full-year estimate are not completed results. The report includes manufacturing, supporting industries, logistics and energy infrastructure among its policy tasks. These are official policy directions without procurement lists for specific wafer, packaging/test, server or factory equipment. GDP growth, consumer inflation and labor productivity have distinct definitions and are not alternative measures of one industry’s growth. US$1.11 trillion is stored as 1,110 USD billion; no base is reverse-calculated from rounded rates, and the full-year estimate is not labelled an actual statistic. Implementation and industry-level demand remain uncertain. Merchandise trade sums exports and imports and cannot be equated with new domestic orders. Location: Report location: a National Assembly session in Hanoi, Vietnam.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>46312</v>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>For industrial-power, data-center-power and measurement/control suppliers, macroeconomic policy provides context for factory and infrastructure customers. Relevant checks concern specific customers’ approved projects, power supply and acceptance schedules; GDP targets and trade estimates alone do not establish equipment demand or purchase orders.</t>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>For precision-power, measurement and control suppliers, automotive regulation, satellite power control and factory logic are specific related applications. Questions concern each product’s tape-out, test and customer-validation stage; combined sales potential cannot establish equipment demand or orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="194" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Singapore’s September NODX rises 68.4%, with exports to Taiwan up 96.9%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Enterprise Singapore reported on October 16 that September non-oil domestic exports rose 68.4% year on year, including a 96.9% rise to Taiwan. Electronic NODX grew 107.6%, but the overall surge also reflected lumpy ship-structure exports and a low prior-year base, rather than AI-chip demand alone. The official report identifies disk media, specialized machinery and ICs among the drivers of NODX to Taiwan; the latter two rose 115.6% and 36.2% year on year. These are product-category trade-value changes without named toolmakers, fabs or end customers. Non-electronic NODX rose 54.2%, with ship structures a major contributor; the agency omitted their growth rate because the prior-year base was exceptionally low. January–September NODX grew 27.6%, a cumulative period distinct from the single-month rate. These are nominal exports and do not isolate price, volume or product-mix effects. Specialized machinery is not broken down into semiconductor tools or individual customer purchases.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>For precision-power and measurement/control suppliers, machinery and IC exports to Taiwan provide aggregate evidence of cross-border manufacturing activity. Questions concern machinery subcategories, prices, physical shipments and customer acceptance timing; nominal growth and ship-structure base effects cannot establish equipment orders.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(news): publish 2026-10-20 daily brief
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-18-en.xlsx
+++ b/docs/exports/week-2026-10-18-en.xlsx
@@ -523,7 +523,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="82" customHeight="1">
+    <row r="3" ht="98" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>01</t>
@@ -538,24 +538,24 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Vietnam–EFTA signature sets out equipment and investment rules, subject to effective terms
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Vietnam and the four EFTA states signed in Hanoi on October 18, covering goods, services, investment, origin and procurement. Machinery and electrical goods are established trade categories, while effective dates and product treatment cannot be established from signature alone.</t>
+            <t xml:space="preserve">AI facilities and servers: separate operating, contract and investment disclosures
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Bitdeer’s October 19 update reports 95% September group GPU utilization, with Malaysia A201 awaiting staged delivery in 2027; Aolani separately announces non-binding LOIs for up to 500 MW. MiTAC discloses a roughly NT$12.62 billion Taiwan manufacturing plan; no supply relationship among the three is stated, and planned capacity is not live capacity.</t>
           </r>
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>46313</v>
-      </c>
-    </row>
-    <row r="4" ht="82" customHeight="1">
+        <v>46314</v>
+      </c>
+    </row>
+    <row r="4" ht="118" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>02</t>
@@ -570,24 +570,26 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Kumamoto fab approval and local equipment-service acquisition authorization
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Professional reports describe Japan’s October 16 approval of JASM’s initial 3nm phase, while Taiwan Mask changed the proposed TCK buyer to the parent. Wafer capacity remains planned and the acquisition has no confirmed closing, with limited direct access to the underlying approval and filing.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>46311</v>
-      </c>
-    </row>
-    <row r="5" ht="102" customHeight="1">
+            <t xml:space="preserve">Wafers, equipment services and packaging have separate approval, investment and validation milestones
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Professional reports describe JASM’s October 16 revised-plan approval and Taiwan Mask’s TCK acquisition authorization, with limited direct access to originals. On October 19, TPK outlines a two-year NT$6 billion TGV plan and PTI reports about NT$739 million in period equipment purchases; plans, authorization and purchases are distinct from production or closing.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Oct 16, Oct 19</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="98" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>03</t>
@@ -602,21 +604,21 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Foxconn’s proposed half-stake in Mitsubishi Electric Mobility covers powertrains and control
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>The October 16 agreement sets ¥115 billion for 50%, against total equity value of ¥230 billion. Closing is planned for October 1, 2027 subject to approvals and conditions, without incremental shipments or factory-output figures.</t>
+            <t xml:space="preserve">PCB equipment purchases in Thailand and academic cooperation in Taiwan
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Zhen Ding’s October 19 disclosure covers about NT$1.086 billion of Thai equipment transactions over nearly a year, not one day of investment, checked through a filing reproduction. NCU separately signs a combined NT$60 million teaching and research partnership with four PCB firms; new capacity and enrollment are unspecified.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="6" ht="82" customHeight="1">
@@ -634,16 +636,16 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Taiwanese storage, fuel logistics and wind works have separate completion milestones
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Foxconn’s partners announced a planned 306 kWh cabinet and H1 2027 supply target on October 16; MOEA said October 18 that CPC began next-quarter fuel procurement. Four installed offshore turbines are a reported official figure, distinct from grid connection or a final loan-repayment settlement.</t>
+            <t xml:space="preserve">Vietnam’s trade signature and Singapore’s exports describe rules and demand separately
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Vietnam and four EFTA states signed an FTA on October 18, with product preferences and effective dates subject to definitive terms. Singapore’s October 16 release reports September NODX growth of 68.4% and Taiwan-bound growth of 96.9%; lumpy ship-structure exports and base effects prevent an AI-only explanation.</t>
           </r>
         </is>
       </c>
@@ -653,7 +655,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="102" customHeight="1">
+    <row r="7" ht="82" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>05</t>
@@ -668,16 +670,16 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Singapore electronics exports and Malaysian chip launches describe shipments and development
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Singapore reported September NODX growth of 68.4% and Taiwan-bound growth of 96.9% on October 16, with ship-structure base effects in the aggregate. Malaysia launched six domestic innovations the same day; RM300 million sales potential lacks a period, and launch-venue reports differ.</t>
+            <t xml:space="preserve">Foxconn proposes half of Mitsubishi Electric Mobility, subject to closing conditions
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>The agreement announced October 16 values the proposed 50% stake at ¥115 billion and covers the automotive-equipment business. Closing is planned for October 1, 2027 subject to approvals and contractual conditions, without incremental orders or factory-output figures.</t>
           </r>
         </is>
       </c>
@@ -701,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -739,7 +741,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="230" customHeight="1">
+    <row r="3" ht="226" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>01</t>
@@ -754,29 +756,29 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Vietnam signs FTA with four EFTA states covering industrial goods, origin and investment rules
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Vietnam and Switzerland, Norway, Iceland and Liechtenstein signed an FTA in Hanoi on October 18, covering goods, services, origin, investment and procurement. Electrical and mechanical machinery already feature in bilateral trade; signature does not establish immediate duty-free treatment for every product. EFTA identifies electrical and mechanical machinery in existing bilateral goods trade. MOIT lists tariffs, technical barriers, customs procedures and investment among the agreement’s provisions, without naming suppliers or newly committed production lines. Negotiations concluded on July 2, followed by signature on October 18. EFTA’s linked chapter factsheet remains the July version and describes product-specific origin rules; signature, domestic procedures and effective preferences are separate stages. The inspected announcements do not establish an entry-into-force date or product-level preference schedules. Equipment tariff, origin and certification treatment depends on the definitive agreement and schedules. Location: Signing location: Hanoi, Vietnam. The inspected official announcements do not identify the venue.</t>
+            <t xml:space="preserve">Bitdeer reports 95% September GPU utilization and staged delivery dates for Malaysia A201
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Bitdeer’s October 19 US release, published October 20 in Taiwan, reports September group AI Cloud GPU utilization of 95%, versus 92% in August, with deployed GPUs unchanged at 4,328. Its approximately 21.7 MW A201 project in Johor Bahru has over 70% long-term contract coverage but is not fully live, with separate readiness and deployment milestones. GPU subscriptions connect racks, power conversion, liquid cooling and site power. External subscriptions rose to 4,007 GPUs from 3,998; these are group figures, not Malaysian site totals. A101’s 2.5 MW is listed as live, separately from planned A201 capacity. ARR is approximately US$86 million and backlog US$2.9 billion, versus US$86 million and US$0.9 billion in August. ARR annualizes month-end daily contracted GPU revenue; backlog is future contractual revenue, not recognized annual sales. A201 lists January 2027 readiness and April full deployment, with over 100 GB300 NVL72 racks procured. Figures are unaudited company disclosures. Acceptance definitions for January readiness versus April go-live, actual energization and revenue-recognition timing are not fully explained. Location: Project site: A201 data center, Johor Bahru, Malaysia; the release also lists Malaysian A101 as live.</t>
           </r>
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>For precision-power and measurement/control suppliers, the relevant link is cross-border trade in Vietnamese factory equipment and test products. Questions concern tariff classification, origin and certification under the effective text; no customer purchasing data establish incremental orders from signature alone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="214" customHeight="1">
+          <t>For power-conversion and measurement suppliers, A201 rack procurement, liquid cooling and energization acceptance raise separate questions. Group utilization cannot substitute for Malaysian load testing; rack installation, power quality and customer acceptance remain unverified, so planned MW alone do not establish equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="194" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>02</t>
@@ -791,6 +793,80 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
+            <t xml:space="preserve">Aolani signs non-binding LOIs for up to 500 MW in Malaysia
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Singapore-based Aolani announced October 19 that it signed LOIs for up to 500 MW of AI data-center capacity across Malaysian sites, targeting service from H2 2027. The LOIs are non-binding and subject to definitive agreements; cities, power conditions and investment value remain undisclosed. Aolani would provide AI infrastructure, GPU deployment and operating requirements. Sites are designed to Tier III standards, not stated as certified. It reports approximately 80 MW committed in 2026 and targets up to 580 MW by 2027, neither equivalent to live capacity or incremental capacity alone. Its site and TNGlobal date the news October 19; ACCESS lists October 18 at 23:45 without a time zone or signing date. The LOIs are non-binding. Counterparties, sites, definitive contracts, approved power, live capacity and signing date remain undisclosed. Location: Project sites: multiple locations in Malaysia, with cities and sites undisclosed; announcement issued in Singapore.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>For data-center power-conversion, distribution-measurement and cooling-control suppliers, the intended sites, owners and GPU operating roles require identification. With power approvals, rack specifications and acceptance schedules undisclosed, the 500 MW intention does not establish equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="210" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">MiTAC’s NT$12.62 billion Taiwan plan covers a new Yangmei plant and two expansions
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Invest Taiwan disclosed MiTAC Computing’s approximately NT$12.62 billion plan on October 19 for a new Yangmei plant and expansion in Zhunan and Linkou, with 300 planned domestic jobs. The official text dates approval to October 16; completion and production-start dates were not disclosed. MiTAC Computing, part of MiTAC Holdings, supplies data-center and enterprise servers. The release describes rack and AI-cluster integration, OCP architecture, air and liquid cooling, and planned AIoT, warehouse logistics, automated assembly and machine vision. The plan includes an enterprise AI computing center, energy management and solar power; LEED Gold is an aspiration, not an awarded certification. NT$12.62 billion is the overall plan, without site allocations or current spending totals. Economic Daily dates approval to October 19; the official text’s October 16 is retained as approval, with October 19 as disclosure. Site-level spending, annual server or rack capacity, approved power allocation and completion/start-up dates remain undisclosed. Location: Project sites: new plant in Yangmei, Taoyuan, Taiwan; existing facilities in Zhunan, Miaoli and Linkou, New Taipei.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>For rack-power, cooling-control and factory-measurement suppliers, the product allocation and line specifications at the three sites merit verification. Approval alone does not establish rack power ratings, equipment acceptance requirements or demand timing; planned investment and awarded equipment contracts remain distinct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="214" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
             <t xml:space="preserve">Follow-up: Japan approves revised JASM Kumamoto plan with 6,000 3nm wafers a month initially
 </t>
           </r>
@@ -801,80 +877,6 @@
               <sz val="11"/>
             </rPr>
             <t>Reuters and CNA report that Japan approved a revised plan for TSMC subsidiary JASM’s second Kumamoto fab on October 16, with initial capacity of 6,000 3nm wafers a month. Approval is the new development; the technology shift was announced in February, and the fab remains under construction. JASM is TSMC’s Japanese manufacturing subsidiary, and the second fab adjoins its existing Kumamoto facility. The approval concerns wafer processing and tool deployment; it contains no new HBM, packaging/test or server shipment data. CNA reports production is planned for late 2028. The earlier 48,000-wafer monthly plan covered a different process mix and build scope, so it is not a comparable base for calculating a capacity reduction. The METI approval document was not directly obtained; capacity and timing rely on professional reporting. Tool lists, yields and actual production capability remain undisclosed. Location: Project site: JASM’s second fab in Kumamoto Prefecture, Japan, adjacent to its first fab.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>46311</v>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>For precision-power and measurement suppliers serving etch and deposition, the relevant customers are fabs and process-tool makers. Questions concern 3nm tool qualification, installation and acceptance timing; planned wafer capacity alone cannot establish equipment purchases or supplier orders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="194" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Follow-up: Taiwan Mask names parent as proposed TCK buyer, with a ¥750 million ceiling
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Taiwan Mask’s board on October 16 authorized its chairman to acquire all of Kumamoto equipment-service company TCK for up to ¥750 million, about NT$160 million according to CNA. The proposed buyer changed from subsidiary Guang Ju Holdings in July to Taiwan Mask itself; the confirmed development is board authorization. Taiwan Mask supplies semiconductor masks; Kumamoto-based TCK provides equipment assembly and engineering services. The filing concerns shares in a service business and gives no additional wafer, packaging or test capacity. ¥750 million is an authorization ceiling. CNA’s NT$160 million equivalent is approximate rather than paid consideration; exchange rates and final terms can change the Taiwan-dollar amount. The filing was checked through Cnyes’s reproduction, without direct retrieval from MOPS. The final price, closing date and integration details remain undisclosed. Location: Target location: T.C.K Corporation, Kumamoto City, Japan. The board meeting venue was not disclosed.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>46311</v>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>For process-power and measurement/control suppliers, equipment assembly and local engineering relate to installation, service and acceptance support. Relevant checks include TCK’s tool scope, customer authorizations and quality processes; the share-acquisition authorization does not establish new supply relationships.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="246" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Foxconn proposes ¥115 billion for 50% of Mitsubishi Electric Mobility, with closing planned in 2027
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Foxconn and Mitsubishi Electric announced on October 16 that Foxconn subsidiary Lin Yin plans to acquire 50% of Mitsubishi Electric Mobility for ¥115 billion and jointly operate the automotive-equipment business. Closing is planned for October 1, 2027, subject to regulatory approvals and contractual conditions. Mitsubishi Electric Mobility handles Mitsubishi Electric’s automotive-equipment business. The joint release identifies electric powertrains, software and vehicle control, with Japan-developed EV platforms as a stated direction. These are cooperation plans rather than new semiconductor-process or data-center capacity announcements. The agreement states enterprise value of ¥320 billion and equity value of ¥230 billion; the ¥115 billion consideration represents 50% of equity value. Enterprise value, total equity value and a partial-stake price have different scopes. Figures remain in the announced yen, without an independently assumed Taiwan-dollar conversion. Closing remains conditional on regulatory approvals and contractual requirements. Incremental orders, integrated production volumes and new-factory start-up schedules were not disclosed. Location: Announcement cities: Taipei, Taiwan, and Tokyo, Japan. No new factory site is specified.</t>
           </r>
         </is>
       </c>
@@ -883,11 +885,11 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>For power-conversion and measurement/control suppliers, the relevant products are electric powertrains, vehicle control and their validation systems. Questions concern platform electrical specifications, supplier qualification and production acceptance; the transaction is conditional and contains no equipment purchasing or customer-order data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="226" customHeight="1">
+          <t>For precision-power and measurement suppliers serving etch and deposition, the relevant customers are fabs and process-tool makers. Questions concern 3nm tool qualification, installation and acceptance timing; planned wafer capacity alone cannot establish equipment purchases or supplier orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="194" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>05</t>
@@ -902,16 +904,16 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Foxconn-led storage partnership plans a 306 kWh cabinet and supply in 2027
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Foxconn and Taiwanese storage partners announced an agreement during Energy Taiwan on October 16 for a planned 306 kWh domestically developed behind-the-meter battery cabinet. They target certification and supply in the first half of 2027, and 100 MWh of cumulative deployment in 2027; both remain targets. Foxconn supplies domestic cells, while partners including Rich Electric, Billion Watts and NoonSpare combine manufacturing, engineering and customer service. The company describes standalone DC battery cabinets or systems integrated with a power-conversion system (PCS) and energy-management system (EMS), for commercial/industrial storage and demand management. The 306 kWh figure describes planned energy per cabinet; 100 MWh describes cumulative market deployment targeted for 2027, a different scope and period. Development is planned in 2026, followed by certification and supply in H1 2027, without a comparable installed base. Completed certification, commercial supply and accepted installations have not been disclosed. The 306 kWh figure is stored energy, not PCS output power, which was not stated. Location: Exhibition venue: Taipei Nangang Exhibition Center Hall 1, Taiwan, October 14–16. The release does not specify a separate signing room.</t>
+            <t xml:space="preserve">Follow-up: Taiwan Mask names parent as proposed TCK buyer, with a ¥750 million ceiling
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Taiwan Mask’s board on October 16 authorized its chairman to acquire all of Kumamoto equipment-service company TCK for up to ¥750 million, about NT$160 million according to CNA. The proposed buyer changed from subsidiary Guang Ju Holdings in July to Taiwan Mask itself; the confirmed development is board authorization. Taiwan Mask supplies semiconductor masks; Kumamoto-based TCK provides equipment assembly and engineering services. The filing concerns shares in a service business and gives no additional wafer, packaging or test capacity. ¥750 million is an authorization ceiling. CNA’s NT$160 million equivalent is approximate rather than paid consideration; exchange rates and final terms can change the Taiwan-dollar amount. The filing was checked through Cnyes’s reproduction, without direct retrieval from MOPS. The final price, closing date and integration details remain undisclosed. Location: Target location: T.C.K Corporation, Kumamoto City, Japan. The board meeting venue was not disclosed.</t>
           </r>
         </is>
       </c>
@@ -920,11 +922,11 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>For power-conversion and measurement/control suppliers, relevant customers include battery-system integrators and industrial users, with PCS/EMS interfaces and site acceptance in scope. Questions concern rated power, communications and certification; the energy specification and deployment target do not establish ordered converter quantities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="230" customHeight="1">
+          <t>For process-power and measurement/control suppliers, equipment assembly and local engineering relate to installation, service and acceptance support. Relevant checks include TCK’s tool scope, customer authorizations and quality processes; the share-acquisition authorization does not establish new supply relationships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="226" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>06</t>
@@ -939,136 +941,247 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">MOEA reports four turbines installed at Taipower Phase II as payment and loan disputes continue
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Taiwan’s MOEA said on October 18 that a batch of three turbines was installed at Taipower’s offshore Phase II project on October 16, bringing the cumulative total to four. MOEA said supervised payments cover subcontractors amid Fuwei’s syndicated-loan dispute; installation progress is separate from a final repayment arrangement. MOEA said Fuwei requested Taipower take over turbine installation, with further work subject to weather and safety conditions. Turbine installation is distinct from electrical testing, grid connection and commercial operation, whose dates were not provided. MOEA described Taipower as a third party to Fuwei’s loan dispute and said it was communicating with the lenders. This describes the ministry’s position on payment mechanisms rather than contractual, lender or court findings on rights and obligations. Installation figures rely on CNA’s report of MOEA’s statement, without direct site-acceptance records or contracts. Grid-connection timing, final liability and bank-repayment arrangements remain unconfirmed. Location: Project: Taipower offshore Phase II, Taiwan. This statement does not provide precise worksite coordinates.</t>
+            <t xml:space="preserve">TPK outlines a two-year NT$6 billion TGV plan and a 300 mm glass-panel exhibit
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>TPK said in an October 19 release reported by CNA that it plans NT$6 billion over two years for Taiwanese through-glass-via facilities and lines, and a 300 × 300 mm panel exhibit at TPCA Show. Its Zhongli pilot line is developing samples with packaging companies, targeting core validation by end-2027 and production in 2028. TGV connects glass processing, metal-filled vias, electrical measurement and advanced packaging. TPK cites modeling work with National Tsing Hua University. The 300 mm figure is panel side length, not wafer capacity. An October 15 report already described the pilot line; the new details are the spending plan and exhibits. The organizer places TPCA Show in Nangang Hall 1 on October 20–22, and IMPACT-IAAC in Hall 2 on October 19–22. Spending, validation and production dates are company plans, not completed customer qualification or commercial delivery. The original company release was not directly retrieved. Customer names, production yields, actual spending and completed qualification dates are undisclosed; technical and timing claims remain company statements. Location: Project site: Zhongli pilot facility, Taoyuan, Taiwan. Exhibition venue: Taipei Nangang Exhibition Center Hall 1, floors 1 and 4, October 20–22.</t>
           </r>
         </is>
       </c>
       <c r="C8" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>For process-power, plating-control and electrical-measurement suppliers, glass processing, via filling and panel-level validation raise specification questions. Pilot work and exhibits do not establish production yield, customer acceptance or equipment orders; development qualification and production spending remain separate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="162" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">PTI discloses approximately NT$739 million in Onto packaging-equipment purchases
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>PTI disclosed October 19 that packaging-equipment purchases from Onto Innovation totaled NT$738.55 million over September 30–October 19. The filing reproduced by professional media describes purchases, without delivery, installation, acceptance or assignment to a specific HBM line. PTI’s official packaging materials describe memory and SSD applications, while Onto supplies inspection, metrology and lithography tools. These business descriptions do not identify this equipment batch as Dragonfly G5, HBM or panel-level packaging capacity. The amount spans the disclosed transaction period, not one day, and no year-earlier base is provided. The disclosure was checked through MoneyDJ rather than directly retrieved from MOPS. Models, quantities, sites, delivery/acceptance and incremental capacity remain undisclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>For packaging-tool power and measurement suppliers, equipment models, power interfaces and installation plans merit verification. The seller’s name does not establish the end process or HBM exposure, and the disclosure is insufficient to infer incremental supporting-equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="198" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Zhen Ding’s Thai subsidiary discloses nearly a year of equipment purchases totaling NT$1.086 billion
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Zhen Ding disclosed October 19 that its Thai subsidiary purchased operating equipment from SYMTEK AUTOMATION CHINA, totaling approximately NT$1.086 billion over October 20, 2025–October 19, 2026. This aggregates nearly a year of transactions, not a single day of new investment, and provides no accepted capacity for the equipment. The buyer is PENG SHEN TECHNOLOGY (THAILAND); the exact disclosed value is NT$1,085,742,322, with contract-based payments to a non-related seller. Zhen Ding’s circuit-board business connects materials and process equipment to electronics assembly, but this filing does not assign the equipment to a specific PCB or substrate product. The filing was checked through professional-information reproduction. Models, quantities, installation site, acceptance, capacity and timing of capital inflows remain undisclosed. Location: Project site: Thai subsidiary; the city and facility for this equipment batch were not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>For factory-automation and process-power suppliers, the equipment’s process position, local servicing and acceptance needs require identification. The nearly year-long aggregate lacks models and installation dates, so it does not establish next-period expansion or incremental supply requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="178" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">NCU and four PCB companies sign NT$60 million education and research partnership
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>National Central University signed a partnership in Taoyuan on October 19 with Zhen Ding, Elite Material, Ta Liang and Topoint, with NT$60 million combined support for courses, company programs, internships and joint research. The PCB-materials and precision-process initiative includes a proposed virtual PCB college, rather than new factory capacity. Partners span circuit boards, copper-clad laminate materials, machining equipment and tools. NCU plans interdisciplinary teaching and industry research. Its release on CNA’s submission platform is university-provided material, distinct from CNA’s separate reporting. NT$60 million is the combined amount, not an equal per-company payment or audited disbursement. Enrollment, company-level allocations and actual payments, course launches and research-output schedules remain undisclosed. Location: Signing venue: Luo Jialun Lecture Hall, National Central University, Taoyuan, Taiwan.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>For process-power, precision-control and measurement suppliers, it is worth verifying whether courses cover materials testing, process control and tool validation. Enrollment and research schedules are unavailable, so the support amount does not establish an available workforce or production-ready technology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="230" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Vietnam signs FTA with four EFTA states covering industrial goods, origin and investment rules
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Vietnam and Switzerland, Norway, Iceland and Liechtenstein signed an FTA in Hanoi on October 18, covering goods, services, origin, investment and procurement. Electrical and mechanical machinery already feature in bilateral trade; signature does not establish immediate duty-free treatment for every product. EFTA identifies electrical and mechanical machinery in existing bilateral goods trade. MOIT lists tariffs, technical barriers, customs procedures and investment among the agreement’s provisions, without naming suppliers or newly committed production lines. Negotiations concluded on July 2, followed by signature on October 18. EFTA’s linked chapter factsheet remains the July version and describes product-specific origin rules; signature, domestic procedures and effective preferences are separate stages. The inspected announcements do not establish an entry-into-force date or product-level preference schedules. Equipment tariff, origin and certification treatment depends on the definitive agreement and schedules. Location: Signing location: Hanoi, Vietnam. The inspected official announcements do not identify the venue.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
         <v>46313</v>
       </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>For industrial-power and measurement/control suppliers, relevant stages include post-installation electrical tests, control validation and grid acceptance. Questions concern acceptance criteria and payment mechanisms for equipment and subcontractors; installation counts do not establish cash collection without contracts and final repayment arrangements.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="146" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">MOEA says year-end fuel supply is secured and CPC has begun Q1 2027 procurement
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Taiwan’s MOEA said on October 18 that CPC was arranging alternative fuel sources and shipping schedules and had begun procurement for Q1 2027, with supply assessed as secured through year-end. This is an official assessment of fuel logistics, without detailed sources, cargoes, inventories or purchase prices. MOEA describes CPC sourcing alternatives and maintaining reserves, with Taipower handling generation and electricity dispatch. The statement does not announce a new industrial tariff or guarantee a specific volume to any factory, park or data center. Supply sufficiency is MOEA’s assessment. Cargo-level procurement and arrival records, user outage rates and final power costs were not provided for independent verification.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>46313</v>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>For industrial/data-center-power and measurement/control suppliers, fuel logistics provide context for customer power conditions. Questions concern site-specific grid access, power quality and acceptance criteria; a national supply assessment does not establish a particular site’s reliability or equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="278" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>08</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Malaysia launches six domestic chip innovations spanning AI storage, industrial FPGA and power control
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Malaysia launched six domestic semiconductor innovations at AiSEM in Kuala Lumpur on October 16, spanning AI processors, storage, programmable logic and power control. The economy minister cited combined sales potential of RM300 million without an achievement period; production shipment figures were not provided. The Edge lists SkyeChip’s MARS1000 AI processor, MaiStorage’s aiDAPTIV+ storage solution, SiliconX’s industrial/automotive FPGA, Infinecs’ automotive power regulator, Weeroc Space’s satellite power controller and Alphaswift’s FC Mini flight controller. Applications extend to factories, computers, servers, vehicles and aerospace. The state-government English report quotes the chief minister saying Weeroc Space’s GaN power chip completed its second tape-out. Tape-out, launch, customer qualification and volume production are separate milestones; RM300 million is the minister’s combined commercial-potential estimate, with no annual revenue or signed orders disclosed. Customer qualification, volume-production timing, sales bases and the period for realizing the combined potential remain undisclosed. Event reports differ between Grand Hyatt and KLCC as the launch venue. Location: Event city: Kuala Lumpur, Malaysia. The organizer schedule, state-government English report and Malay Mail identify Grand Hyatt; the state-government Malay report identifies KLCC, leaving a launch-venue discrepancy.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n">
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>For precision-power and measurement/control suppliers, the relevant link is cross-border trade in Vietnamese factory equipment and test products. Questions concern tariff classification, origin and certification under the effective text; no customer purchasing data establish incremental orders from signature alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="194" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Singapore’s September NODX rises 68.4%, with exports to Taiwan up 96.9%
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Enterprise Singapore reported on October 16 that September non-oil domestic exports rose 68.4% year on year, including a 96.9% rise to Taiwan. Electronic NODX grew 107.6%, but the overall surge also reflected lumpy ship-structure exports and a low prior-year base, rather than AI-chip demand alone. The official report identifies disk media, specialized machinery and ICs among the drivers of NODX to Taiwan; the latter two rose 115.6% and 36.2% year on year. These are product-category trade-value changes without named toolmakers, fabs or end customers. Non-electronic NODX rose 54.2%, with ship structures a major contributor; the agency omitted their growth rate because the prior-year base was exceptionally low. January–September NODX grew 27.6%, a cumulative period distinct from the single-month rate. These are nominal exports and do not isolate price, volume or product-mix effects. Specialized machinery is not broken down into semiconductor tools or individual customer purchases.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
         <v>46311</v>
       </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>For precision-power, measurement and control suppliers, automotive regulation, satellite power control and factory logic are specific related applications. Questions concern each product’s tape-out, test and customer-validation stage; combined sales potential cannot establish equipment demand or orders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="194" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>09</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Singapore’s September NODX rises 68.4%, with exports to Taiwan up 96.9%
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Enterprise Singapore reported on October 16 that September non-oil domestic exports rose 68.4% year on year, including a 96.9% rise to Taiwan. Electronic NODX grew 107.6%, but the overall surge also reflected lumpy ship-structure exports and a low prior-year base, rather than AI-chip demand alone. The official report identifies disk media, specialized machinery and ICs among the drivers of NODX to Taiwan; the latter two rose 115.6% and 36.2% year on year. These are product-category trade-value changes without named toolmakers, fabs or end customers. Non-electronic NODX rose 54.2%, with ship structures a major contributor; the agency omitted their growth rate because the prior-year base was exceptionally low. January–September NODX grew 27.6%, a cumulative period distinct from the single-month rate. These are nominal exports and do not isolate price, volume or product-mix effects. Specialized machinery is not broken down into semiconductor tools or individual customer purchases.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n">
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>For precision-power and measurement/control suppliers, machinery and IC exports to Taiwan provide aggregate evidence of cross-border manufacturing activity. Questions concern machinery subcategories, prices, physical shipments and customer acceptance timing; nominal growth and ship-structure base effects cannot establish equipment orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="246" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Foxconn proposes ¥115 billion for 50% of Mitsubishi Electric Mobility, with closing planned in 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Foxconn and Mitsubishi Electric announced on October 16 that Foxconn subsidiary Lin Yin plans to acquire 50% of Mitsubishi Electric Mobility for ¥115 billion and jointly operate the automotive-equipment business. Closing is planned for October 1, 2027, subject to regulatory approvals and contractual conditions. Mitsubishi Electric Mobility handles Mitsubishi Electric’s automotive-equipment business. The joint release identifies electric powertrains, software and vehicle control, with Japan-developed EV platforms as a stated direction. These are cooperation plans rather than new semiconductor-process or data-center capacity announcements. The agreement states enterprise value of ¥320 billion and equity value of ¥230 billion; the ¥115 billion consideration represents 50% of equity value. Enterprise value, total equity value and a partial-stake price have different scopes. Figures remain in the announced yen, without an independently assumed Taiwan-dollar conversion. Closing remains conditional on regulatory approvals and contractual requirements. Incremental orders, integrated production volumes and new-factory start-up schedules were not disclosed. Location: Announcement cities: Taipei, Taiwan, and Tokyo, Japan. No new factory site is specified.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
         <v>46311</v>
       </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>For precision-power and measurement/control suppliers, machinery and IC exports to Taiwan provide aggregate evidence of cross-border manufacturing activity. Questions concern machinery subcategories, prices, physical shipments and customer acceptance timing; nominal growth and ship-structure base effects cannot establish equipment orders.</t>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>For power-conversion and measurement/control suppliers, the relevant products are electric powertrains, vehicle control and their validation systems. Questions concern platform electrical specifications, supplier qualification and production acceptance; the transaction is conditional and contains no equipment purchasing or customer-order data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(news): publish 2026-10-21 daily brief
Backfill the missed 2026-10-21 daily edition and update the week digest plus export manifests/files.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-18-en.xlsx
+++ b/docs/exports/week-2026-10-18-en.xlsx
@@ -21,8 +21,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="mmm d"/>
+    <numFmt numFmtId="164" formatCode="mmm d"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -119,7 +119,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -551,8 +551,10 @@
           </r>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
-        <v>46314</v>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Oct 19, Oct 20</t>
+        </is>
       </c>
     </row>
     <row r="4" ht="118" customHeight="1">
@@ -703,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -852,7 +854,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="214" customHeight="1">
+    <row r="6" ht="226" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>04</t>
@@ -867,6 +869,43 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
+            <t xml:space="preserve">Malaysia AI-facility commitments and delivery milestones remain distinct
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Bitdeer’s A201 in Malaysia still distinguishes site readiness in January 2027 from full deployment in April 2027, while Aolani’s disclosure is only a non-binding LOI covering up to 500 MW. Both cases show that AI-facility progress is measured separately by contracted coverage, site completion and power readiness, and cannot be treated as installed capacity. The critical milestones for an AI facility span GPUs, server racks, liquid cooling and site power. Company updates list an operating A101, a planned A201, group GPU utilization and future contracted revenue at the same time, which are distinct layers rather than one single operational figure. Bitdeer reports 95% September GPU utilization, but that does not equal A201’s actual monthly output; A201 still distinguishes readiness from full deployment. Aolani lists non-binding LOIs for up to 500 MW, which means the final customer uptake and power timeline are not yet defined. Public disclosure does not yet fully explain A201’s delivery conditions, which customers are already committed, or the gap between energization and revenue recognition. Those items remain contingent on formal delivery notices, power-availability statements and contractual terms. Location: Johor Bahru, Malaysia; A201 and A101 sites listed separately.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>46315</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>For precision-power and measurement-equipment suppliers, the focus is not a single utilization number but whether the site can be delivered, energized and validated. If customer take-up and power milestones remain unresolved, equipment-purchase timing can be delayed, and those points must be checked alongside contract terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="214" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
             <t xml:space="preserve">Follow-up: Japan approves revised JASM Kumamoto plan with 6,000 3nm wafers a month initially
 </t>
           </r>
@@ -877,43 +916,6 @@
               <sz val="11"/>
             </rPr>
             <t>Reuters and CNA report that Japan approved a revised plan for TSMC subsidiary JASM’s second Kumamoto fab on October 16, with initial capacity of 6,000 3nm wafers a month. Approval is the new development; the technology shift was announced in February, and the fab remains under construction. JASM is TSMC’s Japanese manufacturing subsidiary, and the second fab adjoins its existing Kumamoto facility. The approval concerns wafer processing and tool deployment; it contains no new HBM, packaging/test or server shipment data. CNA reports production is planned for late 2028. The earlier 48,000-wafer monthly plan covered a different process mix and build scope, so it is not a comparable base for calculating a capacity reduction. The METI approval document was not directly obtained; capacity and timing rely on professional reporting. Tool lists, yields and actual production capability remain undisclosed. Location: Project site: JASM’s second fab in Kumamoto Prefecture, Japan, adjacent to its first fab.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>46311</v>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>For precision-power and measurement suppliers serving etch and deposition, the relevant customers are fabs and process-tool makers. Questions concern 3nm tool qualification, installation and acceptance timing; planned wafer capacity alone cannot establish equipment purchases or supplier orders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="194" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Follow-up: Taiwan Mask names parent as proposed TCK buyer, with a ¥750 million ceiling
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Taiwan Mask’s board on October 16 authorized its chairman to acquire all of Kumamoto equipment-service company TCK for up to ¥750 million, about NT$160 million according to CNA. The proposed buyer changed from subsidiary Guang Ju Holdings in July to Taiwan Mask itself; the confirmed development is board authorization. Taiwan Mask supplies semiconductor masks; Kumamoto-based TCK provides equipment assembly and engineering services. The filing concerns shares in a service business and gives no additional wafer, packaging or test capacity. ¥750 million is an authorization ceiling. CNA’s NT$160 million equivalent is approximate rather than paid consideration; exchange rates and final terms can change the Taiwan-dollar amount. The filing was checked through Cnyes’s reproduction, without direct retrieval from MOPS. The final price, closing date and integration details remain undisclosed. Location: Target location: T.C.K Corporation, Kumamoto City, Japan. The board meeting venue was not disclosed.</t>
           </r>
         </is>
       </c>
@@ -922,17 +924,54 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
+          <t>For precision-power and measurement suppliers serving etch and deposition, the relevant customers are fabs and process-tool makers. Questions concern 3nm tool qualification, installation and acceptance timing; planned wafer capacity alone cannot establish equipment purchases or supplier orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="194" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Follow-up: Taiwan Mask names parent as proposed TCK buyer, with a ¥750 million ceiling
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Taiwan Mask’s board on October 16 authorized its chairman to acquire all of Kumamoto equipment-service company TCK for up to ¥750 million, about NT$160 million according to CNA. The proposed buyer changed from subsidiary Guang Ju Holdings in July to Taiwan Mask itself; the confirmed development is board authorization. Taiwan Mask supplies semiconductor masks; Kumamoto-based TCK provides equipment assembly and engineering services. The filing concerns shares in a service business and gives no additional wafer, packaging or test capacity. ¥750 million is an authorization ceiling. CNA’s NT$160 million equivalent is approximate rather than paid consideration; exchange rates and final terms can change the Taiwan-dollar amount. The filing was checked through Cnyes’s reproduction, without direct retrieval from MOPS. The final price, closing date and integration details remain undisclosed. Location: Target location: T.C.K Corporation, Kumamoto City, Japan. The board meeting venue was not disclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
           <t>For process-power and measurement/control suppliers, equipment assembly and local engineering relate to installation, service and acceptance support. Relevant checks include TCK’s tool scope, customer authorizations and quality processes; the share-acquisition authorization does not establish new supply relationships.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="226" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+    <row r="9" ht="226" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -951,43 +990,6 @@
               <sz val="11"/>
             </rPr>
             <t>TPK said in an October 19 release reported by CNA that it plans NT$6 billion over two years for Taiwanese through-glass-via facilities and lines, and a 300 × 300 mm panel exhibit at TPCA Show. Its Zhongli pilot line is developing samples with packaging companies, targeting core validation by end-2027 and production in 2028. TGV connects glass processing, metal-filled vias, electrical measurement and advanced packaging. TPK cites modeling work with National Tsing Hua University. The 300 mm figure is panel side length, not wafer capacity. An October 15 report already described the pilot line; the new details are the spending plan and exhibits. The organizer places TPCA Show in Nangang Hall 1 on October 20–22, and IMPACT-IAAC in Hall 2 on October 19–22. Spending, validation and production dates are company plans, not completed customer qualification or commercial delivery. The original company release was not directly retrieved. Customer names, production yields, actual spending and completed qualification dates are undisclosed; technical and timing claims remain company statements. Location: Project site: Zhongli pilot facility, Taoyuan, Taiwan. Exhibition venue: Taipei Nangang Exhibition Center Hall 1, floors 1 and 4, October 20–22.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>46314</v>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>For process-power, plating-control and electrical-measurement suppliers, glass processing, via filling and panel-level validation raise specification questions. Pilot work and exhibits do not establish production yield, customer acceptance or equipment orders; development qualification and production spending remain separate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="162" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">PTI discloses approximately NT$739 million in Onto packaging-equipment purchases
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>PTI disclosed October 19 that packaging-equipment purchases from Onto Innovation totaled NT$738.55 million over September 30–October 19. The filing reproduced by professional media describes purchases, without delivery, installation, acceptance or assignment to a specific HBM line. PTI’s official packaging materials describe memory and SSD applications, while Onto supplies inspection, metrology and lithography tools. These business descriptions do not identify this equipment batch as Dragonfly G5, HBM or panel-level packaging capacity. The amount spans the disclosed transaction period, not one day, and no year-earlier base is provided. The disclosure was checked through MoneyDJ rather than directly retrieved from MOPS. Models, quantities, sites, delivery/acceptance and incremental capacity remain undisclosed.</t>
           </r>
         </is>
       </c>
@@ -996,11 +998,11 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>For packaging-tool power and measurement suppliers, equipment models, power interfaces and installation plans merit verification. The seller’s name does not establish the end process or HBM exposure, and the disclosure is insufficient to infer incremental supporting-equipment demand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="198" customHeight="1">
+          <t>For process-power, plating-control and electrical-measurement suppliers, glass processing, via filling and panel-level validation raise specification questions. Pilot work and exhibits do not establish production yield, customer acceptance or equipment orders; development qualification and production spending remain separate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="162" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>08</t>
@@ -1015,16 +1017,16 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">Zhen Ding’s Thai subsidiary discloses nearly a year of equipment purchases totaling NT$1.086 billion
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Zhen Ding disclosed October 19 that its Thai subsidiary purchased operating equipment from SYMTEK AUTOMATION CHINA, totaling approximately NT$1.086 billion over October 20, 2025–October 19, 2026. This aggregates nearly a year of transactions, not a single day of new investment, and provides no accepted capacity for the equipment. The buyer is PENG SHEN TECHNOLOGY (THAILAND); the exact disclosed value is NT$1,085,742,322, with contract-based payments to a non-related seller. Zhen Ding’s circuit-board business connects materials and process equipment to electronics assembly, but this filing does not assign the equipment to a specific PCB or substrate product. The filing was checked through professional-information reproduction. Models, quantities, installation site, acceptance, capacity and timing of capital inflows remain undisclosed. Location: Project site: Thai subsidiary; the city and facility for this equipment batch were not disclosed.</t>
+            <t xml:space="preserve">PTI discloses approximately NT$739 million in Onto packaging-equipment purchases
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>PTI disclosed October 19 that packaging-equipment purchases from Onto Innovation totaled NT$738.55 million over September 30–October 19. The filing reproduced by professional media describes purchases, without delivery, installation, acceptance or assignment to a specific HBM line. PTI’s official packaging materials describe memory and SSD applications, while Onto supplies inspection, metrology and lithography tools. These business descriptions do not identify this equipment batch as Dragonfly G5, HBM or panel-level packaging capacity. The amount spans the disclosed transaction period, not one day, and no year-earlier base is provided. The disclosure was checked through MoneyDJ rather than directly retrieved from MOPS. Models, quantities, sites, delivery/acceptance and incremental capacity remain undisclosed.</t>
           </r>
         </is>
       </c>
@@ -1033,11 +1035,11 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>For factory-automation and process-power suppliers, the equipment’s process position, local servicing and acceptance needs require identification. The nearly year-long aggregate lacks models and installation dates, so it does not establish next-period expansion or incremental supply requirements.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="178" customHeight="1">
+          <t>For packaging-tool power and measurement suppliers, equipment models, power interfaces and installation plans merit verification. The seller’s name does not establish the end process or HBM exposure, and the disclosure is insufficient to infer incremental supporting-equipment demand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="198" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>09</t>
@@ -1052,16 +1054,16 @@
               <color rgb="0014322B"/>
               <sz val="13"/>
             </rPr>
-            <t xml:space="preserve">NCU and four PCB companies sign NT$60 million education and research partnership
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>National Central University signed a partnership in Taoyuan on October 19 with Zhen Ding, Elite Material, Ta Liang and Topoint, with NT$60 million combined support for courses, company programs, internships and joint research. The PCB-materials and precision-process initiative includes a proposed virtual PCB college, rather than new factory capacity. Partners span circuit boards, copper-clad laminate materials, machining equipment and tools. NCU plans interdisciplinary teaching and industry research. Its release on CNA’s submission platform is university-provided material, distinct from CNA’s separate reporting. NT$60 million is the combined amount, not an equal per-company payment or audited disbursement. Enrollment, company-level allocations and actual payments, course launches and research-output schedules remain undisclosed. Location: Signing venue: Luo Jialun Lecture Hall, National Central University, Taoyuan, Taiwan.</t>
+            <t xml:space="preserve">Zhen Ding’s Thai subsidiary discloses nearly a year of equipment purchases totaling NT$1.086 billion
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Zhen Ding disclosed October 19 that its Thai subsidiary purchased operating equipment from SYMTEK AUTOMATION CHINA, totaling approximately NT$1.086 billion over October 20, 2025–October 19, 2026. This aggregates nearly a year of transactions, not a single day of new investment, and provides no accepted capacity for the equipment. The buyer is PENG SHEN TECHNOLOGY (THAILAND); the exact disclosed value is NT$1,085,742,322, with contract-based payments to a non-related seller. Zhen Ding’s circuit-board business connects materials and process equipment to electronics assembly, but this filing does not assign the equipment to a specific PCB or substrate product. The filing was checked through professional-information reproduction. Models, quantities, installation site, acceptance, capacity and timing of capital inflows remain undisclosed. Location: Project site: Thai subsidiary; the city and facility for this equipment batch were not disclosed.</t>
           </r>
         </is>
       </c>
@@ -1070,17 +1072,54 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
+          <t>For factory-automation and process-power suppliers, the equipment’s process position, local servicing and acceptance needs require identification. The nearly year-long aggregate lacks models and installation dates, so it does not establish next-period expansion or incremental supply requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="178" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">NCU and four PCB companies sign NT$60 million education and research partnership
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>National Central University signed a partnership in Taoyuan on October 19 with Zhen Ding, Elite Material, Ta Liang and Topoint, with NT$60 million combined support for courses, company programs, internships and joint research. The PCB-materials and precision-process initiative includes a proposed virtual PCB college, rather than new factory capacity. Partners span circuit boards, copper-clad laminate materials, machining equipment and tools. NCU plans interdisciplinary teaching and industry research. Its release on CNA’s submission platform is university-provided material, distinct from CNA’s separate reporting. NT$60 million is the combined amount, not an equal per-company payment or audited disbursement. Enrollment, company-level allocations and actual payments, course launches and research-output schedules remain undisclosed. Location: Signing venue: Luo Jialun Lecture Hall, National Central University, Taoyuan, Taiwan.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>46314</v>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
           <t>For process-power, precision-control and measurement suppliers, it is worth verifying whether courses cover materials testing, process control and tool validation. Enrollment and research schedules are unavailable, so the support amount does not establish an available workforce or production-ready technology.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="230" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
+    <row r="13" ht="230" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1102,22 +1141,22 @@
           </r>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C13" s="6" t="n">
         <v>46313</v>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>For precision-power and measurement/control suppliers, the relevant link is cross-border trade in Vietnamese factory equipment and test products. Questions concern tariff classification, origin and certification under the effective text; no customer purchasing data establish incremental orders from signature alone.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="194" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
+    <row r="14" ht="194" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1136,43 +1175,6 @@
               <sz val="11"/>
             </rPr>
             <t>Enterprise Singapore reported on October 16 that September non-oil domestic exports rose 68.4% year on year, including a 96.9% rise to Taiwan. Electronic NODX grew 107.6%, but the overall surge also reflected lumpy ship-structure exports and a low prior-year base, rather than AI-chip demand alone. The official report identifies disk media, specialized machinery and ICs among the drivers of NODX to Taiwan; the latter two rose 115.6% and 36.2% year on year. These are product-category trade-value changes without named toolmakers, fabs or end customers. Non-electronic NODX rose 54.2%, with ship structures a major contributor; the agency omitted their growth rate because the prior-year base was exceptionally low. January–September NODX grew 27.6%, a cumulative period distinct from the single-month rate. These are nominal exports and do not isolate price, volume or product-mix effects. Specialized machinery is not broken down into semiconductor tools or individual customer purchases.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>46311</v>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>For precision-power and measurement/control suppliers, machinery and IC exports to Taiwan provide aggregate evidence of cross-border manufacturing activity. Questions concern machinery subcategories, prices, physical shipments and customer acceptance timing; nominal growth and ship-structure base effects cannot establish equipment orders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="246" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <b val="1"/>
-              <color rgb="0014322B"/>
-              <sz val="13"/>
-            </rPr>
-            <t xml:space="preserve">Foxconn proposes ¥115 billion for 50% of Mitsubishi Electric Mobility, with closing planned in 2027
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Calibri"/>
-              <color rgb="003B4A44"/>
-              <sz val="11"/>
-            </rPr>
-            <t>Foxconn and Mitsubishi Electric announced on October 16 that Foxconn subsidiary Lin Yin plans to acquire 50% of Mitsubishi Electric Mobility for ¥115 billion and jointly operate the automotive-equipment business. Closing is planned for October 1, 2027, subject to regulatory approvals and contractual conditions. Mitsubishi Electric Mobility handles Mitsubishi Electric’s automotive-equipment business. The joint release identifies electric powertrains, software and vehicle control, with Japan-developed EV platforms as a stated direction. These are cooperation plans rather than new semiconductor-process or data-center capacity announcements. The agreement states enterprise value of ¥320 billion and equity value of ¥230 billion; the ¥115 billion consideration represents 50% of equity value. Enterprise value, total equity value and a partial-stake price have different scopes. Figures remain in the announced yen, without an independently assumed Taiwan-dollar conversion. Closing remains conditional on regulatory approvals and contractual requirements. Incremental orders, integrated production volumes and new-factory start-up schedules were not disclosed. Location: Announcement cities: Taipei, Taiwan, and Tokyo, Japan. No new factory site is specified.</t>
           </r>
         </is>
       </c>
@@ -1180,6 +1182,43 @@
         <v>46311</v>
       </c>
       <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>For precision-power and measurement/control suppliers, machinery and IC exports to Taiwan provide aggregate evidence of cross-border manufacturing activity. Questions concern machinery subcategories, prices, physical shipments and customer acceptance timing; nominal growth and ship-structure base effects cannot establish equipment orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="246" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <b val="1"/>
+              <color rgb="0014322B"/>
+              <sz val="13"/>
+            </rPr>
+            <t xml:space="preserve">Foxconn proposes ¥115 billion for 50% of Mitsubishi Electric Mobility, with closing planned in 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <color rgb="003B4A44"/>
+              <sz val="11"/>
+            </rPr>
+            <t>Foxconn and Mitsubishi Electric announced on October 16 that Foxconn subsidiary Lin Yin plans to acquire 50% of Mitsubishi Electric Mobility for ¥115 billion and jointly operate the automotive-equipment business. Closing is planned for October 1, 2027, subject to regulatory approvals and contractual conditions. Mitsubishi Electric Mobility handles Mitsubishi Electric’s automotive-equipment business. The joint release identifies electric powertrains, software and vehicle control, with Japan-developed EV platforms as a stated direction. These are cooperation plans rather than new semiconductor-process or data-center capacity announcements. The agreement states enterprise value of ¥320 billion and equity value of ¥230 billion; the ¥115 billion consideration represents 50% of equity value. Enterprise value, total equity value and a partial-stake price have different scopes. Figures remain in the announced yen, without an independently assumed Taiwan-dollar conversion. Closing remains conditional on regulatory approvals and contractual requirements. Incremental orders, integrated production volumes and new-factory start-up schedules were not disclosed. Location: Announcement cities: Taipei, Taiwan, and Tokyo, Japan. No new factory site is specified.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>For power-conversion and measurement/control suppliers, the relevant products are electric powertrains, vehicle control and their validation systems. Questions concern platform electrical specifications, supplier qualification and production acceptance; the transaction is conditional and contains no equipment purchasing or customer-order data.</t>
         </is>

</xml_diff>

<commit_message>
feat(news): publish 2026-10-24 daily brief
</commit_message>
<xml_diff>
--- a/docs/exports/week-2026-10-18-en.xlsx
+++ b/docs/exports/week-2026-10-18-en.xlsx
@@ -119,7 +119,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="150" customHeight="1">
+    <row r="3" ht="134" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">01</t>
@@ -134,16 +134,16 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Advanced packaging and interconnect: substrates, optical engines, silicon capacitors and materials
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan industry disclosures added capacity and qualification milestones for substrates, testing, CPO optical engines and silicon capacitors. SPIL targets a 15-fold optical-engine increase by mid-2027 and AP Memory completed initial Gen2D wafer validation, while Malaysian and Thai materials expansions remain subject to qualification and actual output.</t>
+            <t xml:space="preserve">Advanced packaging, testing and interconnect: equipment and materials
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">This week's coverage includes substrates, silicon capacitors, optical engines, test equipment and packaging materials. Hermes Testing authorized NT$6.4B for R&amp;D and probe-card equipment facilities on October 22, while KYEC advances and SPIL multiplier targets are separate plans without published qualified shipment volumes.</t>
           </r>
         </is>
       </c>
@@ -168,26 +168,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Wafer production and electronics demand: orders, exports and electric load
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan's September export orders reached US$114.21 billion, Malaysia's exports grew 54.5% year-on-year, and the Taiwan Research Institute reported 11.55% growth in semiconductor electricity use. Geography, bases and definitions differ; power consumption cannot be converted directly into wafer shipments.</t>
+            <t xml:space="preserve">Foundry and electronics demand: orders, exports and September output
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's September orders reached US$114.21B, manufacturing output rose 20.21% and IC output 26.51% in figures released October 23; Malaysia's exports increased 54.5%. Manufacturing missed the previous index range, while orders, production and electricity use remain distinct statistical measures.</t>
           </r>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 16, Oct 19, Oct 20, Oct 21</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="134" customHeight="1">
+          <t xml:space="preserve">Oct 16, Oct 19, Oct 20, Oct 21, Oct 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="114" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">03</t>
@@ -202,26 +202,26 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Memory: Micron labor developments and Malaysia-Japan ZAM design collaboration
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Micron reached a Taichung union agreement on October 21 and 11 Taoyuan union officers began strike action on October 22, when Micron also detailed compensation changes. Malaysia's SkyeChip joined Japan's SAIMEMORY memory architecture R&amp;D, without prototype yield or production timing disclosures.</t>
+            <t xml:space="preserve">Memory supply: Micron negotiations and Malaysia-Japan design
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Micron reached a Taichung union agreement on October 21; Taoyuan union officers struck on October 22, and the union reported 1,633 ballots against Micron's proposal on October 23, moving talks to October 27. Separately, Malaysia's SkyeChip joined SAIMEMORY memory architecture development without production data.</t>
           </r>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 20, Oct 21, Oct 22</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="114" customHeight="1">
+          <t xml:space="preserve">Oct 20, Oct 21, Oct 22, Oct 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="134" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">04</t>
@@ -236,22 +236,22 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">AI data-center systems: Taiwan ODMs and modular deployment
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">MiTAC's Taiwan factory program, Southeast Asian site plans and NVIDIA's modular DSX POD reference design represent distinct stages. Taiwan partners include Foxconn, Delta, GIGABYTE, Pegatron, QCT and Wistron, while the 14-day prepared-site target is an estimate rather than installed data-center capacity.</t>
+            <t xml:space="preserve">Data centers and chip systems: Taiwan ODMs, CPUs and Singapore event
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">This week's developments span MiTAC expansion, data-center facilities, NVIDIA's modular design, Egis-SiPearl CPU-chiplet cooperation and 33 Taiwanese startups heading to Singapore. Technology agreements, delivery targets and planned investment meetings do not represent comparable live capacity.</t>
           </r>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oct 19, Oct 21</t>
+          <t xml:space="preserve">Oct 19, Oct 21, Oct 22, Oct 23</t>
         </is>
       </c>
     </row>
@@ -270,16 +270,16 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Capacity execution: construction, tool materials, talent and power
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Four workers died at TSMC's Kaohsiung F22 site, prompting suspension of similar work, and Reuters separately reported preliminary, unconfirmed inquiries into rare-earth alternatives for fab motors. Singapore's manufacturing-AI support and Malaysia's semiconductor training approvals are program measures, distinct from commissioned factory capacity.</t>
+            <t xml:space="preserve">Factory execution: safety, power, materials and export controls
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Similar steel work was suspended after the TSMC Kaohsiung site accident, with separate reporting on alternative motor materials. AIDC commissioned a 9MW / 54MWh microgrid on October 22, and Taiwan's trade authority added 343 controlled entities, each requiring distinct technical, construction and regulatory interpretation.</t>
           </r>
         </is>
       </c>
@@ -742,7 +742,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="294" customHeight="1">
+    <row r="14" ht="310" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">12</t>
@@ -757,6 +757,43 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Hermes Testing Systems authorizes NT$6.4B for R&amp;D and probe-card manufacturing
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Hermes Testing Systems announced on October 22 that its board authorized two projects totaling NT$6.4 billion, covering a Hsinchu R&amp;D center and a central/southern Taiwan manufacturing center. The latter includes silicon photonics tools, MEMS and thin-film probe cards, reflow equipment and laser probe cleaners, with actual spending contingent on execution. MEMS probe cards are interfaces for wafer-level electrical testing, while silicon photonics assembly tools support optical packaging and testing. The board authorization is not evidence of equipment delivery or commissioning. The R&amp;D center building and fit-out budget is capped at NT$1.5 billion, with NT$3.7 billion for the manufacturing building and NT$1.2 billion for equipment. The chairman has delegated flexibility of up to 10% of the aggregate budget. The manufacturing site's exact city and address, construction start and equipment acceptance dates were not disclosed. Location: Hsinchu, Taiwan (planned R&amp;D center), and central/southern Taiwan (proposed manufacturing center); specific sites undisclosed.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C14" s="6">
+        <v>46317</v>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Test-power, metrology and probe-card tool suppliers would check production specifications, line configurations, acceptance milestones and actual capital disbursement. The authorization does not identify binding equipment purchase orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="294" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">Singapore’s September NODX rises 68.4%, with exports to Taiwan up 96.9%
 </t>
           </r>
@@ -770,22 +807,22 @@
           </r>
         </is>
       </c>
-      <c r="C14" s="6">
+      <c r="C15" s="6">
         <v>46311</v>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">For precision-power and measurement/control suppliers, machinery and IC exports to Taiwan provide aggregate evidence of cross-border manufacturing activity. Questions concern machinery subcategories, prices, physical shipments and customer acceptance timing; nominal growth and ship-structure base effects cannot establish equipment orders.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="306" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+    <row r="16" ht="306" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -807,22 +844,22 @@
           </r>
         </is>
       </c>
-      <c r="C15" s="6">
+      <c r="C16" s="6">
         <v>46315</v>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Precision-power and metrology suppliers would separate ICT, electronics and optical-equipment orders and ask which end products and production lines generated them. The aggregate release does not identify customer allocations, fabrication locations or purchase schedules.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="310" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
+    <row r="17" ht="310" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -844,22 +881,22 @@
           </r>
         </is>
       </c>
-      <c r="C16" s="6">
+      <c r="C17" s="6">
         <v>46314</v>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Precision-power, test and industrial-metrology suppliers would distinguish domestic exports from re-exports and examine equipment and packaging-related tariff lines. The aggregate trade totals do not establish individual OSAT utilization or customer orders.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="262" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
+    <row r="18" ht="262" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -881,22 +918,59 @@
           </r>
         </is>
       </c>
-      <c r="C17" s="6">
+      <c r="C18" s="6">
         <v>46316</v>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Fab power, distribution and metrology suppliers would distinguish utilization changes from new-line commissioning and check load profiles and power-quality requirements. One month's electricity data cannot establish equipment procurement timing.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="326" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">16</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
+    <row r="19" ht="310" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan September manufacturing output rises 20.21% YoY but misses forecast on server mix
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's Ministry of Economic Affairs reported on October 23 a September manufacturing production index of 143.31, up 20.21% year on year, and an industrial index of 140.76, up 19.17%. Integrated circuits rose 26.51% and computer, electronic and optical products 45.92%, but manufacturing came in below the original 146.03–150.03 range, partly because of a change in server product mix. Wafer foundry, DRAM, IC assembly/test and substrates contribute to electronic component manufacturing, up 23.62% year on year. Machinery and equipment output increased 26.02%, partly associated with semiconductor process and test capacity investment. The ministry reported a 15.38% monthly decline in computer, electronic and optical output, contributing to the overall forecast miss. Year-on-year growth and month-on-month contraction use distinct comparison periods. The 141.56–145.86 October manufacturing range is a forecast. Wafer shipments, order breakdown and server model mix were not disclosed, and the original full ministry tables were not directly retrieved.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C19" s="6">
+        <v>46318</v>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process-power, test-equipment and server-power suppliers would examine whether output changes reflect utilization or product mix and how server configuration affects factory loads. Aggregate indices do not reveal specific equipment orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="326" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -918,22 +992,22 @@
           </r>
         </is>
       </c>
-      <c r="C18" s="6">
+      <c r="C20" s="6">
         <v>46315</v>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Test, metrology and process-power suppliers would distinguish operational exposure at Taoyuan and Taichung, including equipment support and new-product qualification. The strike has not yet occurred and no verified production loss supports a procurement inference.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="358" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
+    <row r="21" ht="358" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">19</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -952,80 +1026,6 @@
               <color rgb="FF3B4A44"/>
             </rPr>
             <t xml:space="preserve">Reuters reported on October 21 that Micron and its Taichung union signed an agreement and withdrew from mediation scheduled for October 22, without disclosing terms. The Taoyuan union said talks produced no specific profit-sharing figures and maintained a 24-hour strike plan from 9 a.m. outside the Taoyuan site; Taoyuan focuses on front-end DRAM wafer production, while Taichung covers advanced DRAM, HBM, packaging and testing, but participation and output effects remain unknown. A TrendForce analyst told Reuters that Taoyuan mainly handles front-end DRAM wafer manufacturing, while Taichung produces advanced DRAM and HBM and performs packaging and testing. Any supply effect depends on affected lines and staff and whether maintenance, process monitoring and abnormality handling continue. The Taichung agreement and Taoyuan strike are separate labor processes. Micron said it remained hopeful dialogue would continue; at the Reuters publication time, the Taoyuan action had not begun, so a planned 24-hour strike is not equivalent to 24 hours of lost production. The Taichung agreement terms, actual Taoyuan participation, affected lines, work-in-process handling, yields and shipment schedules were not disclosed. Location: Outside Micron's Taoyuan site, Taiwan (planned strike location as reported by Reuters).</t>
-          </r>
-        </is>
-      </c>
-      <c r="C19" s="6">
-        <v>46316</v>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">For semiconductor process-power, metrology and test-equipment suppliers, the next questions are actual Taoyuan staffing, affected tools and work-in-process nodes, and whether the Taichung agreement covers critical technical staff. Current evidence is insufficient to infer changes in DRAM, HBM or packaging-and-test equipment demand or service schedules.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="294" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">18</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Follow-up: 11 Micron Taoyuan union officers strike as company details quarterly bonuses
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Eleven Micron Taoyuan union officers began a 24-hour strike at 9 a.m. on October 22, a day after the separate Taichung union reached an agreement. Micron announced quarterly profit-linked bonuses paid half in cash and half in equity, raised Taiwan retirement contributions from 8% to 10% and added three paid-leave days; production effects were not disclosed. Taoyuan is linked to front-end DRAM manufacturing, while Taichung covers advanced DRAM, HBM and packaging/test. Participation by union officers does not establish a fab-wide shutdown or a specific wafer loss. Micron management said cash payments will follow quarterly results while equity vests after one year. The company also described shift-allowance and salary changes, while Taoyuan union representatives maintained negotiations remain open. No fab utilization, shipment loss, Taoyuan union acceptance or full Taichung settlement terms were disclosed. Location: Outside Micron's Taoyuan site, Taiwan (reported union action location).</t>
-          </r>
-        </is>
-      </c>
-      <c r="C20" s="6">
-        <v>46317</v>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Process-power and memory-test suppliers would verify shift coverage, maintenance and work-in-process status, and any concrete schedule effects from talks. Eleven union officers' participation alone does not quantify tool demand or yield changes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="262" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">19</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Malaysia's SkyeChip joins Japan's SAIMEMORY ZAM memory design program
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Japan's SAIMEMORY and Malaysia's SkyeChip announced a design-engineering engagement on October 21 for Z-Angle Memory (ZAM) targeting AI data centers. SkyeChip will contribute silicon design, memory-interface engineering and custom IP; prototype validation, bandwidth and commercialization dates were not disclosed. SAIMEMORY is a SoftBank subsidiary developing a high-capacity, high-bandwidth memory architecture; SkyeChip provides memory IP design and integration. This is a development engagement, without evidence of a completed HBM manufacturing line. The work is associated with a Japan NEDO-subsidized Post-5G infrastructure R&amp;D project. The statement covers engineering support and eventual commercialization intentions, without product specifications or fab investment figures. ZAM prototype yield, bandwidth, measured power, customer samples and volume-production timing remain unknown.</t>
           </r>
         </is>
       </c>
@@ -1034,17 +1034,128 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">For semiconductor process-power, metrology and test-equipment suppliers, the next questions are actual Taoyuan staffing, affected tools and work-in-process nodes, and whether the Taichung agreement covers critical technical staff. Current evidence is insufficient to infer changes in DRAM, HBM or packaging-and-test equipment demand or service schedules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="294" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Follow-up: 11 Micron Taoyuan union officers strike as company details quarterly bonuses
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Eleven Micron Taoyuan union officers began a 24-hour strike at 9 a.m. on October 22, a day after the separate Taichung union reached an agreement. Micron announced quarterly profit-linked bonuses paid half in cash and half in equity, raised Taiwan retirement contributions from 8% to 10% and added three paid-leave days; production effects were not disclosed. Taoyuan is linked to front-end DRAM manufacturing, while Taichung covers advanced DRAM, HBM and packaging/test. Participation by union officers does not establish a fab-wide shutdown or a specific wafer loss. Micron management said cash payments will follow quarterly results while equity vests after one year. The company also described shift-allowance and salary changes, while Taoyuan union representatives maintained negotiations remain open. No fab utilization, shipment loss, Taoyuan union acceptance or full Taichung settlement terms were disclosed. Location: Outside Micron's Taoyuan site, Taiwan (reported union action location).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C22" s="6">
+        <v>46317</v>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Process-power and memory-test suppliers would verify shift coverage, maintenance and work-in-process status, and any concrete schedule effects from talks. Eleven union officers' participation alone does not quantify tool demand or yield changes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="262" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Malaysia's SkyeChip joins Japan's SAIMEMORY ZAM memory design program
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Japan's SAIMEMORY and Malaysia's SkyeChip announced a design-engineering engagement on October 21 for Z-Angle Memory (ZAM) targeting AI data centers. SkyeChip will contribute silicon design, memory-interface engineering and custom IP; prototype validation, bandwidth and commercialization dates were not disclosed. SAIMEMORY is a SoftBank subsidiary developing a high-capacity, high-bandwidth memory architecture; SkyeChip provides memory IP design and integration. This is a development engagement, without evidence of a completed HBM manufacturing line. The work is associated with a Japan NEDO-subsidized Post-5G infrastructure R&amp;D project. The statement covers engineering support and eventual commercialization intentions, without product specifications or fab investment figures. ZAM prototype yield, bandwidth, measured power, customer samples and volume-production timing remain unknown.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C23" s="6">
+        <v>46316</v>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Memory power, test and interface suppliers would need ZAM voltage, bandwidth, packaging and qualification specifications. There is no evidence yet of sample production or test-capacity demand.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="342" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
+    <row r="24" ht="262" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Follow-up: 1,633 Micron Taoyuan union members oppose plan; talks move to Oct 27
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">On October 23, Micron's Taoyuan union reported 1,637 ballots on the company's revised compensation plan, of which 1,633 rejected it, about 70% of all union members according to the union. Talks originally scheduled for October 23 were postponed to October 27 because of the typhoon; no production-loss figures were disclosed. Taoyuan is associated with front-end DRAM fabrication. A 24-hour action by 11 union officers began October 22 and ended at 9 a.m. October 23. The new development is the membership ballot and rescheduled meeting, not another strike. Micron had proposed quarterly bonuses, shift allowances and higher retirement contributions. The union said 1,633 rejections represented roughly 99% of votes cast but around 70% of total membership, which are different denominators. Full membership rolls, meeting transcripts and quantified effects on output, yield or deliveries were not available.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C24" s="6">
+        <v>46318</v>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Memory process-power and testing suppliers would track the rescheduled negotiation and actual technical staffing. A membership ballot does not quantify utilization or shipment impacts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="342" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">23</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1066,22 +1177,22 @@
           </r>
         </is>
       </c>
-      <c r="C22" s="6">
+      <c r="C25" s="6">
         <v>46314</v>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">For power-conversion and measurement suppliers, A201 rack procurement, liquid cooling and energization acceptance raise separate questions. Group utilization cannot substitute for Malaysian load testing; rack installation, power quality and customer acceptance remain unverified, so planned MW alone do not establish equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="326" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">21</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
+    <row r="26" ht="326" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1103,22 +1214,22 @@
           </r>
         </is>
       </c>
-      <c r="C23" s="6">
+      <c r="C26" s="6">
         <v>46314</v>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">For rack-power, cooling-control and factory-measurement suppliers, the product allocation and line specifications at the three sites merit verification. Approval alone does not establish rack power ratings, equipment acceptance requirements or demand timing; planned investment and awarded equipment contracts remain distinct.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="258" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
+    <row r="27" ht="258" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1140,22 +1251,22 @@
           </r>
         </is>
       </c>
-      <c r="C24" s="6">
+      <c r="C27" s="6">
         <v>46314</v>
       </c>
-      <c r="D24" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">For data-center power-conversion, distribution-measurement and cooling-control suppliers, the intended sites, owners and GPU operating roles require identification. With power approvals, rack specifications and acceptance schedules undisclosed, the 500 MW intention does not establish equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="374" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
+    <row r="28" ht="374" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1177,22 +1288,22 @@
           </r>
         </is>
       </c>
-      <c r="C25" s="6">
+      <c r="C28" s="6">
         <v>46316</v>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">For data-center power, network-monitoring and test-equipment suppliers, the key question is whether cooperation extends to cable landing stations, backup power, fault location and repair coordination rather than policy dialogue alone. There is no budget, procurement or technical specification from which to infer new equipment demand.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="310" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">24</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
+    <row r="29" ht="310" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">27</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1214,127 +1325,16 @@
           </r>
         </is>
       </c>
-      <c r="C26" s="6">
+      <c r="C29" s="6">
         <v>46316</v>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Data-center power, CDU and rack test suppliers would verify factory acceptance scope, on-site power and cooling interfaces and partner responsibilities. The minimum deployment duration remains an estimate without observed installation results.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="358" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">25</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Foxconn-led storage partnership plans a 306 kWh cabinet and supply in 2027
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Foxconn and Taiwanese storage partners announced an agreement during Energy Taiwan on October 16 for a planned 306 kWh domestically developed behind-the-meter battery cabinet. They target certification and supply in the first half of 2027, and 100 MWh of cumulative deployment in 2027; both remain targets. Foxconn supplies domestic cells, while partners including Rich Electric, Billion Watts and NoonSpare combine manufacturing, engineering and customer service. The company describes standalone DC battery cabinets or systems integrated with a power-conversion system (PCS) and energy-management system (EMS), for commercial/industrial storage and demand management. The 306 kWh figure describes planned energy per cabinet; 100 MWh describes cumulative market deployment targeted for 2027, a different scope and period. Development is planned in 2026, followed by certification and supply in H1 2027, without a comparable installed base. Completed certification, commercial supply and accepted installations have not been disclosed. The 306 kWh figure is stored energy, not PCS output power, which was not stated. Location: Exhibition venue: Taipei Nangang Exhibition Center Hall 1, Taiwan, October 14–16. The release does not specify a separate signing room.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C27" s="6">
-        <v>46311</v>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">For power-conversion and measurement/control suppliers, relevant customers include battery-system integrators and industrial users, with PCS/EMS interfaces and site acceptance in scope. Questions concern rated power, communications and certification; the energy specification and deployment target do not establish ordered converter quantities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="326" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">26</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">MOEA reports four turbines installed at Taipower Phase II as payment and loan disputes continue
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan’s MOEA said on October 18 that a batch of three turbines was installed at Taipower’s offshore Phase II project on October 16, bringing the cumulative total to four. MOEA said supervised payments cover subcontractors amid Fuwei’s syndicated-loan dispute; installation progress is separate from a final repayment arrangement. MOEA said Fuwei requested Taipower take over turbine installation, with further work subject to weather and safety conditions. Turbine installation is distinct from electrical testing, grid connection and commercial operation, whose dates were not provided. MOEA described Taipower as a third party to Fuwei’s loan dispute and said it was communicating with the lenders. This describes the ministry’s position on payment mechanisms rather than contractual, lender or court findings on rights and obligations. Installation figures rely on CNA’s report of MOEA’s statement, without direct site-acceptance records or contracts. Grid-connection timing, final liability and bank-repayment arrangements remain unconfirmed. Location: Project: Taipower offshore Phase II, Taiwan. This statement does not provide precise worksite coordinates.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C28" s="6">
-        <v>46313</v>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">For industrial-power and measurement/control suppliers, relevant stages include post-installation electrical tests, control validation and grid acceptance. Questions concern acceptance criteria and payment mechanisms for equipment and subcontractors; installation counts do not establish cash collection without contracts and final repayment arrangements.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="390" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">27</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <b/>
-              <sz val="13"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF14322B"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan investment forum signs 13 foreign-company LOIs; 27 proposals total about NT$666 billion
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan's MOEA said at its October 20 investment forum in Taipei that 27 prospective investors represented about NT$666 billion in proposals, and 13 companies signed letters of intent. The total spans semiconductors and non-technology services, so it represents plans and expressions of intent rather than approved, funded or completed factory spending. MOEA said the 13 LOI signatories proposed about NT$62.1 billion of future investment, a subset of the roughly NT$666 billion across 27 prospective investors. Named participants included BASF expanding its Guanyin chemicals facility for advanced processes, Qnity planning capacity and about 200 additional jobs, Canon Semiconductor Equipment planning a Taiwan training center, and Lam Research expanding local R&amp;D. Execution dates and expenditure schedules require project-level confirmation. MOEA separately cited US$19.23 billion in inward investment for January–September 2026, a different measure that cannot be added to forward-looking LOIs. The NT$62.1 billion represented by the 13 signatories remains planned investment subject to approvals, binding contracts and spending schedules; the portfolio also includes non-technology services. Project-level industries, sites, comparable investment periods and conversion of the 13 LOIs into binding investment were not fully disclosed. Location: Taipei Nangang Exhibition Center Hall 2, 7F Rooms 701C/D, Taiwan; forum venue, not project sites.</t>
-          </r>
-        </is>
-      </c>
-      <c r="C29" s="6">
-        <v>46315</v>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Precision-power, measurement and control suppliers would seek project-level identification of wafer-fab, packaging or factory-automation plans and their contractual status. The NT$666 billion is not broken down by project or delivery milestone and cannot establish equipment orders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="358" customHeight="1">
+    <row r="30" ht="242" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">28</t>
@@ -1349,29 +1349,29 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">Taiwan's TAITRONICS industry pavilion displays 65 results and announces Dutch-port cooperation
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan's Industrial Development Administration showcased 65 technology results at TAITRONICS &amp; AIoT Taiwan on October 20, claiming associated program output exceeding NT$34.2 billion. Taiwanese firm An-En-Jia signed an AI-vision cooperation memorandum with Dutch company CERTUS Automation; the agency reported a Rotterdam port trial and a formal order, without a breakdown of output across exhibitors. The five zones cover AI chips, next-generation communications, industrial AI, smart displays and startups, linking embedded systems, power electronics and factories. The agency separately reported around NT$7 billion in policy support over three years, a different measure from supported output. According to IDA, An-En-Jia's system completed commercial validation at Kaohsiung Port in 2025, underwent a Rotterdam Port trial in June 2026, and secured a formal order. Full rollout is planned for January 2027, but order value, delivered unit count and acceptance criteria were not disclosed. IDA did not disaggregate the NT$34.2 billion in attributed output by company, product or reporting period; the Rotterdam contract value, installed units and actual field outcomes remain unpublished. Location: Taipei Nangang Exhibition Center Hall 1, Taiwan; TAITRONICS &amp; AIoT Taiwan exhibition venue.</t>
+            <t xml:space="preserve">Taiwan's Egis and French SiPearl sign CPU chiplet collaboration
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's Egis group signed a strategic agreement with French CPU designer SiPearl at its October 22 Tech Day, covering processor technology, chiplet integration and high-performance computing markets. Group company ALi is developing the Mobius100 platform with SiPearl support; no shipment volumes, capital expenditure or validation dates were disclosed. SiPearl is a fabless processor designer, connecting the cooperation with Taiwan chip design, advanced packaging and HPC system supply chains. Signing a framework does not establish product qualification or customer procurement. CNA cited the companies and the Ministry of Economic Affairs on an existing Taiwan-France R&amp;D support framework. Historical 2025 commitments are context and are not contract value for this new agreement. Licensing terms, CPU performance, process node, packaging configuration, test progress and customer names are undisclosed.</t>
           </r>
         </is>
       </c>
       <c r="C30" s="6">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">For power-conversion, metrology and automation suppliers, the Rotterdam order after a trial provides a more concrete commercialization milestone than a demonstration, but the planned 2027 rollout remains distinct from current deployment. Contract value, unit count and procurement terms were not disclosed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="342" customHeight="1">
+          <t xml:space="preserve">Advanced packaging power and server test suppliers would seek Mobius100 qualification, chiplet interface and packaging details. Technical specifications and manufacturing dates remain unannounced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="290" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">29</t>
@@ -1386,25 +1386,25 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
-            <t xml:space="preserve">MOEA demonstrates six smart industrial-safety technologies at Kaohsiung's Linyuan plant
-</t>
-          </r>
-          <r>
-            <rPr>
-              <sz val="11"/>
-              <rFont val="Calibri"/>
-              <color rgb="FF3B4A44"/>
-            </rPr>
-            <t xml:space="preserve">Taiwan's Industrial Development Administration demonstrated six smart industrial-safety applications at Taiwan VCM's Linyuan factory in Kaohsiung on October 20, covering worker location, inspection, VOC analysis, machine vision, pipeline monitoring and factory management. The event documented a pilot implementation, but the agency did not report verified before-and-after fault, downtime or incident rates. Six categories include anomalous-worker detection and location, automated inspections, volatile-organic-compound analysis, people/vehicle imaging, equipment and pipeline monitoring, and factory operations management. They touch sensors, industrial controls and maintenance software, whose qualification criteria differ from semiconductor-production tools. IDA says its smart-safety program began in 2024, with Taiwan VCM participating as a demonstration site. The new October 20 development was the on-site showcase, not the initial installation of all systems. Equipment counts, plant coverage, comparable safety outcomes and rollout budgets across other factories remain undisclosed. Location: Taiwan VCM Linyuan plant, Linyuan District, Kaohsiung, Taiwan; demonstration factory site.</t>
+            <t xml:space="preserve">Taiwan announces 33 startups for Singapore SWITCH event
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's National Development Council said on October 23 it will bring 33 startups to Singapore's SWITCH event from October 27 to 29, its largest delegation yet, spanning semiconductors, robotics, AI and clean energy. Meetings with investors and enterprises are scheduled engagements, not completed investments. SWITCH is a technology innovation event, and Taiwan's planned national pavilion will connect startups with venture funds, industrial firms and research partners. This is an investment ecosystem announcement without new installed factory capacity. CNA reported plans for the Taiwan-Singapore startup forum and Taiwan Tech Connect. The official SWITCH website confirms October 27-29 at Marina Bay Sands Expo &amp; Convention Centre, Halls A-C on Level 1 and ballrooms on Level 3. Investments, customer agreements and technical qualification outcomes for the 33 participating startups have not been disclosed; attendance remains scheduled. Location: Marina Bay Sands Expo &amp; Convention Centre, Halls A-C (Level 1) and ballrooms (Level 3), Singapore (scheduled exhibition and conference venue).</t>
           </r>
         </is>
       </c>
       <c r="C31" s="6">
-        <v>46315</v>
+        <v>46318</v>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Industrial control and metrology suppliers could examine sensing accuracy, false alarms, connectivity and integration with existing factory systems. Installation counts and comparable operating outcomes are not yet published.</t>
+          <t xml:space="preserve">Semiconductor metrology and industrial automation suppliers would look for actual qualification and supplier-adoption outcomes after the event. Only delegation size and activities have been announced.</t>
         </is>
       </c>
     </row>
@@ -1423,6 +1423,191 @@
               <rFont val="Calibri"/>
               <color rgb="FF14322B"/>
             </rPr>
+            <t xml:space="preserve">Foxconn-led storage partnership plans a 306 kWh cabinet and supply in 2027
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Foxconn and Taiwanese storage partners announced an agreement during Energy Taiwan on October 16 for a planned 306 kWh domestically developed behind-the-meter battery cabinet. They target certification and supply in the first half of 2027, and 100 MWh of cumulative deployment in 2027; both remain targets. Foxconn supplies domestic cells, while partners including Rich Electric, Billion Watts and NoonSpare combine manufacturing, engineering and customer service. The company describes standalone DC battery cabinets or systems integrated with a power-conversion system (PCS) and energy-management system (EMS), for commercial/industrial storage and demand management. The 306 kWh figure describes planned energy per cabinet; 100 MWh describes cumulative market deployment targeted for 2027, a different scope and period. Development is planned in 2026, followed by certification and supply in H1 2027, without a comparable installed base. Completed certification, commercial supply and accepted installations have not been disclosed. The 306 kWh figure is stored energy, not PCS output power, which was not stated. Location: Exhibition venue: Taipei Nangang Exhibition Center Hall 1, Taiwan, October 14–16. The release does not specify a separate signing room.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C32" s="6">
+        <v>46311</v>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For power-conversion and measurement/control suppliers, relevant customers include battery-system integrators and industrial users, with PCS/EMS interfaces and site acceptance in scope. Questions concern rated power, communications and certification; the energy specification and deployment target do not establish ordered converter quantities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="326" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">MOEA reports four turbines installed at Taipower Phase II as payment and loan disputes continue
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan’s MOEA said on October 18 that a batch of three turbines was installed at Taipower’s offshore Phase II project on October 16, bringing the cumulative total to four. MOEA said supervised payments cover subcontractors amid Fuwei’s syndicated-loan dispute; installation progress is separate from a final repayment arrangement. MOEA said Fuwei requested Taipower take over turbine installation, with further work subject to weather and safety conditions. Turbine installation is distinct from electrical testing, grid connection and commercial operation, whose dates were not provided. MOEA described Taipower as a third party to Fuwei’s loan dispute and said it was communicating with the lenders. This describes the ministry’s position on payment mechanisms rather than contractual, lender or court findings on rights and obligations. Installation figures rely on CNA’s report of MOEA’s statement, without direct site-acceptance records or contracts. Grid-connection timing, final liability and bank-repayment arrangements remain unconfirmed. Location: Project: Taipower offshore Phase II, Taiwan. This statement does not provide precise worksite coordinates.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C33" s="6">
+        <v>46313</v>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For industrial-power and measurement/control suppliers, relevant stages include post-installation electrical tests, control validation and grid acceptance. Questions concern acceptance criteria and payment mechanisms for equipment and subcontractors; installation counts do not establish cash collection without contracts and final repayment arrangements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="390" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan investment forum signs 13 foreign-company LOIs; 27 proposals total about NT$666 billion
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's MOEA said at its October 20 investment forum in Taipei that 27 prospective investors represented about NT$666 billion in proposals, and 13 companies signed letters of intent. The total spans semiconductors and non-technology services, so it represents plans and expressions of intent rather than approved, funded or completed factory spending. MOEA said the 13 LOI signatories proposed about NT$62.1 billion of future investment, a subset of the roughly NT$666 billion across 27 prospective investors. Named participants included BASF expanding its Guanyin chemicals facility for advanced processes, Qnity planning capacity and about 200 additional jobs, Canon Semiconductor Equipment planning a Taiwan training center, and Lam Research expanding local R&amp;D. Execution dates and expenditure schedules require project-level confirmation. MOEA separately cited US$19.23 billion in inward investment for January–September 2026, a different measure that cannot be added to forward-looking LOIs. The NT$62.1 billion represented by the 13 signatories remains planned investment subject to approvals, binding contracts and spending schedules; the portfolio also includes non-technology services. Project-level industries, sites, comparable investment periods and conversion of the 13 LOIs into binding investment were not fully disclosed. Location: Taipei Nangang Exhibition Center Hall 2, 7F Rooms 701C/D, Taiwan; forum venue, not project sites.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C34" s="6">
+        <v>46315</v>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Precision-power, measurement and control suppliers would seek project-level identification of wafer-fab, packaging or factory-automation plans and their contractual status. The NT$666 billion is not broken down by project or delivery milestone and cannot establish equipment orders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="358" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">33</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's TAITRONICS industry pavilion displays 65 results and announces Dutch-port cooperation
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's Industrial Development Administration showcased 65 technology results at TAITRONICS &amp; AIoT Taiwan on October 20, claiming associated program output exceeding NT$34.2 billion. Taiwanese firm An-En-Jia signed an AI-vision cooperation memorandum with Dutch company CERTUS Automation; the agency reported a Rotterdam port trial and a formal order, without a breakdown of output across exhibitors. The five zones cover AI chips, next-generation communications, industrial AI, smart displays and startups, linking embedded systems, power electronics and factories. The agency separately reported around NT$7 billion in policy support over three years, a different measure from supported output. According to IDA, An-En-Jia's system completed commercial validation at Kaohsiung Port in 2025, underwent a Rotterdam Port trial in June 2026, and secured a formal order. Full rollout is planned for January 2027, but order value, delivered unit count and acceptance criteria were not disclosed. IDA did not disaggregate the NT$34.2 billion in attributed output by company, product or reporting period; the Rotterdam contract value, installed units and actual field outcomes remain unpublished. Location: Taipei Nangang Exhibition Center Hall 1, Taiwan; TAITRONICS &amp; AIoT Taiwan exhibition venue.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C35" s="6">
+        <v>46315</v>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For power-conversion, metrology and automation suppliers, the Rotterdam order after a trial provides a more concrete commercialization milestone than a demonstration, but the planned 2027 rollout remains distinct from current deployment. Contract value, unit count and procurement terms were not disclosed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="342" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">34</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">MOEA demonstrates six smart industrial-safety technologies at Kaohsiung's Linyuan plant
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's Industrial Development Administration demonstrated six smart industrial-safety applications at Taiwan VCM's Linyuan factory in Kaohsiung on October 20, covering worker location, inspection, VOC analysis, machine vision, pipeline monitoring and factory management. The event documented a pilot implementation, but the agency did not report verified before-and-after fault, downtime or incident rates. Six categories include anomalous-worker detection and location, automated inspections, volatile-organic-compound analysis, people/vehicle imaging, equipment and pipeline monitoring, and factory operations management. They touch sensors, industrial controls and maintenance software, whose qualification criteria differ from semiconductor-production tools. IDA says its smart-safety program began in 2024, with Taiwan VCM participating as a demonstration site. The new October 20 development was the on-site showcase, not the initial installation of all systems. Equipment counts, plant coverage, comparable safety outcomes and rollout budgets across other factories remain undisclosed. Location: Taiwan VCM Linyuan plant, Linyuan District, Kaohsiung, Taiwan; demonstration factory site.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C36" s="6">
+        <v>46315</v>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial control and metrology suppliers could examine sensing accuracy, false alarms, connectivity and integration with existing factory systems. Installation counts and comparable operating outcomes are not yet published.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="358" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">35</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
             <t xml:space="preserve">Four workers die at TSMC Kaohsiung F22 site; similar steel work suspended across Taiwan
 </t>
           </r>
@@ -1436,22 +1621,22 @@
           </r>
         </is>
       </c>
-      <c r="C32" s="6">
+      <c r="C37" s="6">
         <v>46315</v>
       </c>
-      <c r="D32" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">For semiconductor equipment and precision-power suppliers, the next checks are which fabs link steel work, utilities and tool move-in on the same critical path and what contractor restart conditions apply. Without suspension duration and move-in milestones, changes to installation, acceptance or service schedules cannot be inferred.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="342" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
+    <row r="38" ht="342" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">36</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1473,22 +1658,22 @@
           </r>
         </is>
       </c>
-      <c r="C33" s="6">
+      <c r="C38" s="6">
         <v>46316</v>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">For precision-manufacturing equipment, measurement and control suppliers, the useful checks are whether grants cover equipment-data integration, predictive maintenance, process control and quotation automation, and the deployment scale of semiconductor use cases. The funding is a policy commitment without beneficiary or procurement lists, so hardware demand cannot yet be inferred.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="278" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">32</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
+    <row r="39" ht="278" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">37</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1510,22 +1695,22 @@
           </r>
         </is>
       </c>
-      <c r="C34" s="6">
+      <c r="C39" s="6">
         <v>46317</v>
       </c>
-      <c r="D34" s="7" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power, motor-drive and controls suppliers would ask whether alternative magnets alter motor efficiency, reliability testing or tool requalification. No rollout or replacement quantities are confirmed.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="278" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">33</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
+    <row r="40" ht="278" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1547,12 +1732,86 @@
           </r>
         </is>
       </c>
-      <c r="C35" s="6">
+      <c r="C40" s="6">
         <v>46317</v>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Process-power, test and automation suppliers would check which courses cover tool operation and related job functions. Approved slots, aggregate completions and job placements use different definitions and cannot establish current hiring capacity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="290" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">39</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">AIDC commissions 9MW / 54MWh industrial microgrid in Taichung
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Aerospace Industrial Development Corporation commissioned a 9MW / 54MWh industrial microgrid at its Shuinan plant in Taichung on October 22, integrating storage, energy management and electrical protection. AIDC claims up to six hours of plant backup and estimates nearly 40% annual energy-cost savings under current tariffs; the savings remain a projection. The behind-the-meter storage system shifts consumption between off-peak and peak periods, with potential integration of wind, solar and backup generation. It involves industrial power conversion, battery management and electrical controls relevant to factory and data-center loads. AIDC describes islanded operation and layered electrical safety systems, using a NT$9.29/kWh summer peak/off-peak tariff differential in its savings model. An earlier 2MW / 2.7MWh demonstration is separate from the new 9MW / 54MWh facility. Full-year realized savings, supplier contract values, system round-trip efficiency and backup test profiles were not disclosed. Location: Shuinan plant, Taichung, Taiwan (commissioned microgrid site).</t>
+          </r>
+        </is>
+      </c>
+      <c r="C41" s="6">
+        <v>46317</v>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial power and storage suppliers would evaluate islanding transition times, load tolerance and peak/off-peak metering. AIDC's 40% cost estimate needs full-year operational evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="246" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="13"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF14322B"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan trade authority adds 343 entities and removes 90 from strategic export list
+</t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+              <color rgb="FF3B4A44"/>
+            </rPr>
+            <t xml:space="preserve">Taiwan's International Trade Administration announced on October 22 the addition of 343 entities and removal of 90 from its strategic high-tech export entity list under Article 13 of the Trade Act. Exports of covered goods to listed recipients require prior authorization, with Customs supporting border enforcement. The strategic high-tech regime can cover dual-use semiconductor tools, electronics, material processing, computing and sensors, subject to product classification, listed end users and end-use rules. The agency says over 11,660 people and entities are now included; newly added entries span Iran, Russia, Mexico, UAE, Türkiye and China, among others. The October 22 list update has been published. The release does not identify affected Taiwan company transactions or sector-specific trade values.</t>
+          </r>
+        </is>
+      </c>
+      <c r="C42" s="6">
+        <v>46317</v>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Equipment and test suppliers would need to distinguish commodity classification, end-use and recipient-list status from granted export permits. The entity count does not quantify changed export revenue.</t>
         </is>
       </c>
     </row>

</xml_diff>